<commit_message>
Resynchronise le gabarit FAD : mise en forme de cellules
Reporte dans backend/src/assets/modele-fad.xlsx les changements de mise
en forme apportés au gabarit source (fonds/couleurs d'en-tête), sans
impact sur la correspondance cellule/champ — tests fadPdfGenerator et
rendu LibreOffice vérifiés.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ForClaude/CDC/Modèle-FAD-XLSX.xlsx
+++ b/ForClaude/CDC/Modèle-FAD-XLSX.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\laure\Developement\Projets\VIGIE\ForClaude\CDC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F336B98D-5C5C-455F-BE2A-956135C4B09A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AAF3BBD-9F04-4F9C-8AE5-4834A4582606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FBD6BC2A-920F-401F-BE14-790DF3E005BB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{FBD6BC2A-920F-401F-BE14-790DF3E005BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Correspondance Cellule-Valeur" sheetId="4" r:id="rId1"/>
@@ -137,9 +137,6 @@
     <t>*</t>
   </si>
   <si>
-    <t>Les prix constitutifs de cette commande sont indiqués le devis joint.</t>
-  </si>
-  <si>
     <t>Cellule</t>
   </si>
   <si>
@@ -638,6 +635,9 @@
   </si>
   <si>
     <t>Si la procédure d'achat=HORS_MARCHE et si motif_choix="Autre" alors libelle_motif_choix  sinon vide</t>
+  </si>
+  <si>
+    <t>Les prix constitutifs de la commande sont indiqués le devis joint.</t>
   </si>
 </sst>
 </file>
@@ -648,7 +648,7 @@
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -766,14 +766,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -845,6 +837,22 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="22"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1102,7 +1110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="195">
+  <cellXfs count="197">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1130,7 +1138,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1188,7 +1196,7 @@
     <xf numFmtId="14" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1200,9 +1208,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1231,14 +1239,356 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="13" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="13" fillId="4" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="20" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1259,414 +1609,80 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="12"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="12"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="12"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="12"/>
+    </xf>
+    <xf numFmtId="44" fontId="21" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="21" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="21" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="13" fillId="4" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="13" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="4" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="22" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2087,667 +2103,667 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>51</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="C3" s="4" t="s">
         <v>54</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="4" t="s">
         <v>57</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>60</v>
-      </c>
       <c r="C5" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>62</v>
-      </c>
       <c r="C6" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>64</v>
-      </c>
       <c r="C7" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>67</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="C10" s="4" t="s">
         <v>70</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>73</v>
-      </c>
       <c r="C11" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>75</v>
-      </c>
       <c r="C12" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="C13" s="4" t="s">
         <v>77</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="C14" s="4" t="s">
         <v>80</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="C15" s="4" t="s">
         <v>83</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>86</v>
-      </c>
       <c r="C16" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="C17" s="4" t="s">
         <v>88</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="C18" s="4" t="s">
         <v>91</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="C20" s="4" t="s">
         <v>96</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="B21" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B21" s="4" t="s">
-        <v>99</v>
-      </c>
       <c r="C21" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="B22" s="4" t="s">
-        <v>101</v>
-      </c>
       <c r="C22" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="B23" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B23" s="4" t="s">
-        <v>103</v>
-      </c>
       <c r="C23" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="B24" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="B24" s="4" t="s">
-        <v>105</v>
-      </c>
       <c r="C24" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="C25" s="4" t="s">
         <v>106</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="C29" s="4" t="s">
         <v>111</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="B30" s="4" t="s">
         <v>113</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="B31" s="4" t="s">
         <v>115</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="B32" s="4" t="s">
         <v>117</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="B33" s="4" t="s">
         <v>119</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="B34" s="4" t="s">
         <v>121</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="B35" s="4" t="s">
         <v>123</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="B36" s="4" t="s">
         <v>125</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="B37" s="4" t="s">
         <v>127</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="B38" s="4" t="s">
         <v>129</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="B39" s="4" t="s">
         <v>131</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="B40" s="4" t="s">
         <v>133</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="B41" s="4" t="s">
         <v>135</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="B42" s="4" t="s">
         <v>137</v>
-      </c>
-      <c r="B42" s="4" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="B43" s="4" t="s">
         <v>139</v>
-      </c>
-      <c r="B43" s="4" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="B44" s="4" t="s">
         <v>141</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="B45" s="4" t="s">
         <v>143</v>
-      </c>
-      <c r="B45" s="4" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="B46" s="4" t="s">
         <v>145</v>
-      </c>
-      <c r="B46" s="4" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
+        <v>146</v>
+      </c>
+      <c r="B47" s="4" t="s">
         <v>147</v>
-      </c>
-      <c r="B47" s="4" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
+        <v>148</v>
+      </c>
+      <c r="B48" s="4" t="s">
         <v>149</v>
-      </c>
-      <c r="B48" s="4" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="B49" s="4" t="s">
         <v>151</v>
-      </c>
-      <c r="B49" s="4" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="B50" s="4" t="s">
         <v>153</v>
-      </c>
-      <c r="B50" s="4" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="B51" s="4" t="s">
         <v>155</v>
-      </c>
-      <c r="B51" s="4" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="B52" s="4" t="s">
         <v>157</v>
-      </c>
-      <c r="B52" s="4" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="B53" s="4" t="s">
         <v>159</v>
-      </c>
-      <c r="B53" s="4" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="B54" s="4" t="s">
         <v>161</v>
-      </c>
-      <c r="B54" s="4" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="B55" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="B55" s="4" t="s">
-        <v>164</v>
-      </c>
       <c r="C55" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="14" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="B57" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="B57" s="4" t="s">
-        <v>167</v>
-      </c>
       <c r="C57" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B58" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C58" s="4" t="s">
         <v>57</v>
-      </c>
-      <c r="C58" s="4" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="14" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="B60" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="B60" s="4" t="s">
-        <v>170</v>
-      </c>
       <c r="C60" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="B61" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="B61" s="4" t="s">
+    </row>
+    <row r="62" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A62" s="14" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="62" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A62" s="14" t="s">
+      <c r="B62" s="48" t="s">
         <v>173</v>
-      </c>
-      <c r="B62" s="49" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="14" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="B64" s="4" t="s">
         <v>175</v>
-      </c>
-      <c r="B64" s="4" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="B65" s="4" t="s">
         <v>177</v>
-      </c>
-      <c r="B65" s="4" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="B66" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="B66" s="4" t="s">
+    </row>
+    <row r="67" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A67" s="14" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="67" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A67" s="14" t="s">
+      <c r="B67" s="48" t="s">
         <v>181</v>
-      </c>
-      <c r="B67" s="49" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="B68" s="4" t="s">
         <v>183</v>
-      </c>
-      <c r="B68" s="4" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" s="14" t="s">
+        <v>184</v>
+      </c>
+      <c r="B69" s="4" t="s">
         <v>185</v>
-      </c>
-      <c r="B69" s="4" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" s="14" t="s">
+        <v>186</v>
+      </c>
+      <c r="B70" s="4" t="s">
         <v>187</v>
-      </c>
-      <c r="B70" s="4" t="s">
-        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -2783,375 +2799,375 @@
   <sheetData>
     <row r="1" spans="1:33" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
-      <c r="B1" s="95"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="96"/>
-      <c r="K1" s="96"/>
-      <c r="L1" s="96"/>
-      <c r="M1" s="97"/>
-      <c r="N1" s="83" t="s">
+      <c r="B1" s="146"/>
+      <c r="C1" s="147"/>
+      <c r="D1" s="147"/>
+      <c r="E1" s="147"/>
+      <c r="F1" s="147"/>
+      <c r="G1" s="147"/>
+      <c r="H1" s="147"/>
+      <c r="I1" s="147"/>
+      <c r="J1" s="147"/>
+      <c r="K1" s="147"/>
+      <c r="L1" s="147"/>
+      <c r="M1" s="148"/>
+      <c r="N1" s="134" t="s">
         <v>0</v>
       </c>
-      <c r="O1" s="84"/>
-      <c r="P1" s="84"/>
-      <c r="Q1" s="84"/>
-      <c r="R1" s="84"/>
-      <c r="S1" s="84"/>
-      <c r="T1" s="84"/>
-      <c r="U1" s="84"/>
-      <c r="V1" s="84"/>
-      <c r="W1" s="84"/>
-      <c r="X1" s="84"/>
-      <c r="Y1" s="84"/>
-      <c r="Z1" s="84"/>
-      <c r="AA1" s="84"/>
-      <c r="AB1" s="84"/>
-      <c r="AC1" s="84"/>
-      <c r="AD1" s="84"/>
-      <c r="AE1" s="84"/>
-      <c r="AF1" s="84"/>
-      <c r="AG1" s="85"/>
+      <c r="O1" s="135"/>
+      <c r="P1" s="135"/>
+      <c r="Q1" s="135"/>
+      <c r="R1" s="135"/>
+      <c r="S1" s="135"/>
+      <c r="T1" s="135"/>
+      <c r="U1" s="135"/>
+      <c r="V1" s="135"/>
+      <c r="W1" s="135"/>
+      <c r="X1" s="135"/>
+      <c r="Y1" s="135"/>
+      <c r="Z1" s="135"/>
+      <c r="AA1" s="135"/>
+      <c r="AB1" s="135"/>
+      <c r="AC1" s="135"/>
+      <c r="AD1" s="135"/>
+      <c r="AE1" s="135"/>
+      <c r="AF1" s="135"/>
+      <c r="AG1" s="136"/>
     </row>
     <row r="2" spans="1:33" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
-      <c r="B2" s="98"/>
-      <c r="C2" s="76"/>
-      <c r="D2" s="76"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="76"/>
-      <c r="G2" s="76"/>
-      <c r="H2" s="76"/>
-      <c r="I2" s="76"/>
-      <c r="J2" s="76"/>
-      <c r="K2" s="76"/>
-      <c r="L2" s="76"/>
-      <c r="M2" s="99"/>
-      <c r="N2" s="86" t="s">
+      <c r="B2" s="149"/>
+      <c r="C2" s="150"/>
+      <c r="D2" s="150"/>
+      <c r="E2" s="150"/>
+      <c r="F2" s="150"/>
+      <c r="G2" s="150"/>
+      <c r="H2" s="150"/>
+      <c r="I2" s="150"/>
+      <c r="J2" s="150"/>
+      <c r="K2" s="150"/>
+      <c r="L2" s="150"/>
+      <c r="M2" s="151"/>
+      <c r="N2" s="137" t="s">
         <v>2</v>
       </c>
-      <c r="O2" s="87"/>
-      <c r="P2" s="87"/>
-      <c r="Q2" s="87"/>
-      <c r="R2" s="87"/>
-      <c r="S2" s="87"/>
-      <c r="T2" s="87"/>
-      <c r="U2" s="87"/>
-      <c r="V2" s="87"/>
-      <c r="W2" s="87"/>
-      <c r="X2" s="87"/>
-      <c r="Y2" s="87"/>
-      <c r="Z2" s="87"/>
-      <c r="AA2" s="87"/>
-      <c r="AB2" s="87"/>
-      <c r="AC2" s="87"/>
-      <c r="AD2" s="87"/>
-      <c r="AE2" s="87"/>
-      <c r="AF2" s="87"/>
-      <c r="AG2" s="88"/>
+      <c r="O2" s="138"/>
+      <c r="P2" s="138"/>
+      <c r="Q2" s="138"/>
+      <c r="R2" s="138"/>
+      <c r="S2" s="138"/>
+      <c r="T2" s="138"/>
+      <c r="U2" s="138"/>
+      <c r="V2" s="138"/>
+      <c r="W2" s="138"/>
+      <c r="X2" s="138"/>
+      <c r="Y2" s="138"/>
+      <c r="Z2" s="138"/>
+      <c r="AA2" s="138"/>
+      <c r="AB2" s="138"/>
+      <c r="AC2" s="138"/>
+      <c r="AD2" s="138"/>
+      <c r="AE2" s="138"/>
+      <c r="AF2" s="138"/>
+      <c r="AG2" s="139"/>
     </row>
     <row r="3" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
-      <c r="B3" s="100"/>
-      <c r="C3" s="101"/>
-      <c r="D3" s="101"/>
-      <c r="E3" s="101"/>
-      <c r="F3" s="101"/>
-      <c r="G3" s="101"/>
-      <c r="H3" s="101"/>
-      <c r="I3" s="101"/>
-      <c r="J3" s="101"/>
-      <c r="K3" s="101"/>
-      <c r="L3" s="101"/>
-      <c r="M3" s="102"/>
-      <c r="N3" s="89" t="s">
+      <c r="B3" s="152"/>
+      <c r="C3" s="153"/>
+      <c r="D3" s="153"/>
+      <c r="E3" s="153"/>
+      <c r="F3" s="153"/>
+      <c r="G3" s="153"/>
+      <c r="H3" s="153"/>
+      <c r="I3" s="153"/>
+      <c r="J3" s="153"/>
+      <c r="K3" s="153"/>
+      <c r="L3" s="153"/>
+      <c r="M3" s="154"/>
+      <c r="N3" s="140" t="s">
         <v>8</v>
       </c>
-      <c r="O3" s="90"/>
-      <c r="P3" s="90"/>
-      <c r="Q3" s="90"/>
-      <c r="R3" s="90"/>
-      <c r="S3" s="90"/>
-      <c r="T3" s="90"/>
-      <c r="U3" s="90"/>
-      <c r="V3" s="90"/>
-      <c r="W3" s="90"/>
-      <c r="X3" s="90"/>
-      <c r="Y3" s="90"/>
-      <c r="Z3" s="90"/>
-      <c r="AA3" s="90"/>
-      <c r="AB3" s="90"/>
-      <c r="AC3" s="90"/>
-      <c r="AD3" s="90"/>
-      <c r="AE3" s="90"/>
-      <c r="AF3" s="90"/>
-      <c r="AG3" s="91"/>
+      <c r="O3" s="141"/>
+      <c r="P3" s="141"/>
+      <c r="Q3" s="141"/>
+      <c r="R3" s="141"/>
+      <c r="S3" s="141"/>
+      <c r="T3" s="141"/>
+      <c r="U3" s="141"/>
+      <c r="V3" s="141"/>
+      <c r="W3" s="141"/>
+      <c r="X3" s="141"/>
+      <c r="Y3" s="141"/>
+      <c r="Z3" s="141"/>
+      <c r="AA3" s="141"/>
+      <c r="AB3" s="141"/>
+      <c r="AC3" s="141"/>
+      <c r="AD3" s="141"/>
+      <c r="AE3" s="141"/>
+      <c r="AF3" s="141"/>
+      <c r="AG3" s="142"/>
     </row>
     <row r="4" spans="1:33" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
-      <c r="B4" s="100"/>
-      <c r="C4" s="101"/>
-      <c r="D4" s="101"/>
-      <c r="E4" s="101"/>
-      <c r="F4" s="101"/>
-      <c r="G4" s="101"/>
-      <c r="H4" s="101"/>
-      <c r="I4" s="101"/>
-      <c r="J4" s="101"/>
-      <c r="K4" s="101"/>
-      <c r="L4" s="101"/>
-      <c r="M4" s="102"/>
-      <c r="N4" s="89"/>
-      <c r="O4" s="90"/>
-      <c r="P4" s="90"/>
-      <c r="Q4" s="90"/>
-      <c r="R4" s="90"/>
-      <c r="S4" s="90"/>
-      <c r="T4" s="90"/>
-      <c r="U4" s="90"/>
-      <c r="V4" s="90"/>
-      <c r="W4" s="90"/>
-      <c r="X4" s="90"/>
-      <c r="Y4" s="90"/>
-      <c r="Z4" s="90"/>
-      <c r="AA4" s="90"/>
-      <c r="AB4" s="90"/>
-      <c r="AC4" s="90"/>
-      <c r="AD4" s="90"/>
-      <c r="AE4" s="90"/>
-      <c r="AF4" s="90"/>
-      <c r="AG4" s="91"/>
+      <c r="B4" s="152"/>
+      <c r="C4" s="153"/>
+      <c r="D4" s="153"/>
+      <c r="E4" s="153"/>
+      <c r="F4" s="153"/>
+      <c r="G4" s="153"/>
+      <c r="H4" s="153"/>
+      <c r="I4" s="153"/>
+      <c r="J4" s="153"/>
+      <c r="K4" s="153"/>
+      <c r="L4" s="153"/>
+      <c r="M4" s="154"/>
+      <c r="N4" s="140"/>
+      <c r="O4" s="141"/>
+      <c r="P4" s="141"/>
+      <c r="Q4" s="141"/>
+      <c r="R4" s="141"/>
+      <c r="S4" s="141"/>
+      <c r="T4" s="141"/>
+      <c r="U4" s="141"/>
+      <c r="V4" s="141"/>
+      <c r="W4" s="141"/>
+      <c r="X4" s="141"/>
+      <c r="Y4" s="141"/>
+      <c r="Z4" s="141"/>
+      <c r="AA4" s="141"/>
+      <c r="AB4" s="141"/>
+      <c r="AC4" s="141"/>
+      <c r="AD4" s="141"/>
+      <c r="AE4" s="141"/>
+      <c r="AF4" s="141"/>
+      <c r="AG4" s="142"/>
     </row>
     <row r="5" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
-      <c r="B5" s="111"/>
-      <c r="C5" s="112"/>
-      <c r="D5" s="112"/>
-      <c r="E5" s="112"/>
-      <c r="F5" s="112"/>
-      <c r="G5" s="112"/>
-      <c r="H5" s="112"/>
-      <c r="I5" s="112"/>
-      <c r="J5" s="112"/>
-      <c r="K5" s="112"/>
-      <c r="L5" s="112"/>
-      <c r="M5" s="113"/>
-      <c r="N5" s="92"/>
-      <c r="O5" s="93"/>
-      <c r="P5" s="93"/>
-      <c r="Q5" s="93"/>
-      <c r="R5" s="93"/>
-      <c r="S5" s="93"/>
-      <c r="T5" s="93"/>
-      <c r="U5" s="93"/>
-      <c r="V5" s="93"/>
-      <c r="W5" s="93"/>
-      <c r="X5" s="93"/>
-      <c r="Y5" s="93"/>
-      <c r="Z5" s="93"/>
-      <c r="AA5" s="93"/>
-      <c r="AB5" s="93"/>
-      <c r="AC5" s="93"/>
-      <c r="AD5" s="93"/>
-      <c r="AE5" s="93"/>
-      <c r="AF5" s="93"/>
-      <c r="AG5" s="94"/>
-    </row>
-    <row r="6" spans="1:33" ht="31.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B5" s="114"/>
+      <c r="C5" s="115"/>
+      <c r="D5" s="115"/>
+      <c r="E5" s="115"/>
+      <c r="F5" s="115"/>
+      <c r="G5" s="115"/>
+      <c r="H5" s="115"/>
+      <c r="I5" s="115"/>
+      <c r="J5" s="115"/>
+      <c r="K5" s="115"/>
+      <c r="L5" s="115"/>
+      <c r="M5" s="116"/>
+      <c r="N5" s="143"/>
+      <c r="O5" s="144"/>
+      <c r="P5" s="144"/>
+      <c r="Q5" s="144"/>
+      <c r="R5" s="144"/>
+      <c r="S5" s="144"/>
+      <c r="T5" s="144"/>
+      <c r="U5" s="144"/>
+      <c r="V5" s="144"/>
+      <c r="W5" s="144"/>
+      <c r="X5" s="144"/>
+      <c r="Y5" s="144"/>
+      <c r="Z5" s="144"/>
+      <c r="AA5" s="144"/>
+      <c r="AB5" s="144"/>
+      <c r="AC5" s="144"/>
+      <c r="AD5" s="144"/>
+      <c r="AE5" s="144"/>
+      <c r="AF5" s="144"/>
+      <c r="AG5" s="145"/>
+    </row>
+    <row r="6" spans="1:33" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
-      <c r="B6" s="104" t="s">
-        <v>32</v>
-      </c>
-      <c r="C6" s="104"/>
-      <c r="D6" s="104"/>
-      <c r="E6" s="104"/>
-      <c r="F6" s="104"/>
-      <c r="G6" s="103"/>
-      <c r="H6" s="103"/>
-      <c r="I6" s="103"/>
-      <c r="J6" s="103"/>
-      <c r="K6" s="103"/>
-      <c r="L6" s="103"/>
-      <c r="M6" s="103"/>
-      <c r="N6" s="103"/>
-      <c r="O6" s="103"/>
-      <c r="P6" s="103"/>
-      <c r="Q6" s="103"/>
-      <c r="R6" s="103"/>
-      <c r="S6" s="103"/>
-      <c r="T6" s="103"/>
-      <c r="U6" s="103"/>
-      <c r="V6" s="103"/>
-      <c r="W6" s="103"/>
-      <c r="X6" s="103"/>
-      <c r="Y6" s="48"/>
-      <c r="Z6" s="48"/>
-      <c r="AA6" s="48"/>
-      <c r="AB6" s="48"/>
-      <c r="AC6" s="48"/>
-      <c r="AD6" s="48"/>
-      <c r="AE6" s="48"/>
-      <c r="AF6" s="48"/>
-      <c r="AG6" s="48"/>
+      <c r="B6" s="155" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="155"/>
+      <c r="D6" s="155"/>
+      <c r="E6" s="155"/>
+      <c r="F6" s="155"/>
+      <c r="G6" s="70"/>
+      <c r="H6" s="70"/>
+      <c r="I6" s="70"/>
+      <c r="J6" s="70"/>
+      <c r="K6" s="70"/>
+      <c r="L6" s="70"/>
+      <c r="M6" s="70"/>
+      <c r="N6" s="70"/>
+      <c r="O6" s="70"/>
+      <c r="P6" s="70"/>
+      <c r="Q6" s="70"/>
+      <c r="R6" s="70"/>
+      <c r="S6" s="70"/>
+      <c r="T6" s="70"/>
+      <c r="U6" s="70"/>
+      <c r="V6" s="70"/>
+      <c r="W6" s="70"/>
+      <c r="X6" s="70"/>
+      <c r="Y6" s="196"/>
+      <c r="Z6" s="196"/>
+      <c r="AA6" s="196"/>
+      <c r="AB6" s="196"/>
+      <c r="AC6" s="196"/>
+      <c r="AD6" s="196"/>
+      <c r="AE6" s="196"/>
+      <c r="AF6" s="196"/>
+      <c r="AG6" s="196"/>
     </row>
     <row r="7" spans="1:33" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
-      <c r="B7" s="104" t="s">
+      <c r="B7" s="155" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="104"/>
-      <c r="D7" s="104"/>
-      <c r="E7" s="104"/>
-      <c r="F7" s="104"/>
-      <c r="G7" s="103"/>
-      <c r="H7" s="103"/>
-      <c r="I7" s="103"/>
-      <c r="J7" s="103"/>
-      <c r="K7" s="103"/>
-      <c r="L7" s="103"/>
-      <c r="M7" s="103"/>
-      <c r="N7" s="103"/>
-      <c r="O7" s="103"/>
-      <c r="P7" s="103"/>
-      <c r="Q7" s="114" t="s">
+      <c r="C7" s="155"/>
+      <c r="D7" s="155"/>
+      <c r="E7" s="155"/>
+      <c r="F7" s="155"/>
+      <c r="G7" s="70"/>
+      <c r="H7" s="70"/>
+      <c r="I7" s="70"/>
+      <c r="J7" s="70"/>
+      <c r="K7" s="70"/>
+      <c r="L7" s="70"/>
+      <c r="M7" s="70"/>
+      <c r="N7" s="70"/>
+      <c r="O7" s="70"/>
+      <c r="P7" s="70"/>
+      <c r="Q7" s="117" t="s">
         <v>10</v>
       </c>
-      <c r="R7" s="114"/>
-      <c r="S7" s="114"/>
-      <c r="T7" s="115"/>
-      <c r="U7" s="115"/>
-      <c r="V7" s="115"/>
-      <c r="W7" s="115"/>
-      <c r="X7" s="115"/>
-      <c r="Y7" s="115"/>
-      <c r="Z7" s="115"/>
-      <c r="AA7" s="115"/>
-      <c r="AB7" s="115"/>
-      <c r="AC7" s="115"/>
-      <c r="AD7" s="115"/>
-      <c r="AE7" s="115"/>
-      <c r="AF7" s="115"/>
-      <c r="AG7" s="115"/>
-    </row>
-    <row r="8" spans="1:33" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="R7" s="117"/>
+      <c r="S7" s="117"/>
+      <c r="T7" s="192"/>
+      <c r="U7" s="192"/>
+      <c r="V7" s="192"/>
+      <c r="W7" s="192"/>
+      <c r="X7" s="192"/>
+      <c r="Y7" s="192"/>
+      <c r="Z7" s="192"/>
+      <c r="AA7" s="192"/>
+      <c r="AB7" s="192"/>
+      <c r="AC7" s="192"/>
+      <c r="AD7" s="192"/>
+      <c r="AE7" s="192"/>
+      <c r="AF7" s="192"/>
+      <c r="AG7" s="192"/>
+    </row>
+    <row r="8" spans="1:33" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
-      <c r="B8" s="68" t="s">
+      <c r="B8" s="156" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="69"/>
-      <c r="D8" s="70"/>
-      <c r="E8" s="71"/>
-      <c r="F8" s="71"/>
-      <c r="G8" s="71"/>
-      <c r="H8" s="71"/>
-      <c r="I8" s="71"/>
-      <c r="J8" s="71"/>
-      <c r="K8" s="71"/>
-      <c r="L8" s="71"/>
-      <c r="M8" s="71"/>
-      <c r="N8" s="71"/>
-      <c r="O8" s="71"/>
-      <c r="P8" s="71"/>
-      <c r="Q8" s="71"/>
-      <c r="R8" s="71"/>
-      <c r="S8" s="71"/>
-      <c r="T8" s="71"/>
-      <c r="U8" s="71"/>
-      <c r="V8" s="71"/>
-      <c r="W8" s="71"/>
-      <c r="X8" s="71"/>
-      <c r="Y8" s="71"/>
-      <c r="Z8" s="71"/>
-      <c r="AA8" s="71"/>
-      <c r="AB8" s="71"/>
-      <c r="AC8" s="71"/>
-      <c r="AD8" s="71"/>
-      <c r="AE8" s="71"/>
-      <c r="AF8" s="71"/>
-      <c r="AG8" s="72"/>
+      <c r="C8" s="157"/>
+      <c r="D8" s="193"/>
+      <c r="E8" s="194"/>
+      <c r="F8" s="194"/>
+      <c r="G8" s="194"/>
+      <c r="H8" s="194"/>
+      <c r="I8" s="194"/>
+      <c r="J8" s="194"/>
+      <c r="K8" s="194"/>
+      <c r="L8" s="194"/>
+      <c r="M8" s="194"/>
+      <c r="N8" s="194"/>
+      <c r="O8" s="194"/>
+      <c r="P8" s="194"/>
+      <c r="Q8" s="194"/>
+      <c r="R8" s="194"/>
+      <c r="S8" s="194"/>
+      <c r="T8" s="194"/>
+      <c r="U8" s="194"/>
+      <c r="V8" s="194"/>
+      <c r="W8" s="194"/>
+      <c r="X8" s="194"/>
+      <c r="Y8" s="194"/>
+      <c r="Z8" s="194"/>
+      <c r="AA8" s="194"/>
+      <c r="AB8" s="194"/>
+      <c r="AC8" s="194"/>
+      <c r="AD8" s="194"/>
+      <c r="AE8" s="194"/>
+      <c r="AF8" s="194"/>
+      <c r="AG8" s="195"/>
     </row>
     <row r="9" spans="1:33" ht="134.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
-      <c r="B9" s="73"/>
-      <c r="C9" s="74"/>
-      <c r="D9" s="74"/>
-      <c r="E9" s="74"/>
-      <c r="F9" s="74"/>
-      <c r="G9" s="74"/>
-      <c r="H9" s="74"/>
-      <c r="I9" s="74"/>
-      <c r="J9" s="74"/>
-      <c r="K9" s="74"/>
-      <c r="L9" s="74"/>
-      <c r="M9" s="74"/>
-      <c r="N9" s="74"/>
-      <c r="O9" s="74"/>
-      <c r="P9" s="74"/>
-      <c r="Q9" s="74"/>
-      <c r="R9" s="74"/>
-      <c r="S9" s="74"/>
-      <c r="T9" s="74"/>
-      <c r="U9" s="74"/>
-      <c r="V9" s="74"/>
-      <c r="W9" s="74"/>
-      <c r="X9" s="74"/>
-      <c r="Y9" s="74"/>
-      <c r="Z9" s="74"/>
-      <c r="AA9" s="74"/>
-      <c r="AB9" s="74"/>
-      <c r="AC9" s="74"/>
-      <c r="AD9" s="74"/>
-      <c r="AE9" s="74"/>
-      <c r="AF9" s="74"/>
-      <c r="AG9" s="75"/>
+      <c r="B9" s="158"/>
+      <c r="C9" s="159"/>
+      <c r="D9" s="159"/>
+      <c r="E9" s="159"/>
+      <c r="F9" s="159"/>
+      <c r="G9" s="159"/>
+      <c r="H9" s="159"/>
+      <c r="I9" s="159"/>
+      <c r="J9" s="159"/>
+      <c r="K9" s="159"/>
+      <c r="L9" s="159"/>
+      <c r="M9" s="159"/>
+      <c r="N9" s="159"/>
+      <c r="O9" s="159"/>
+      <c r="P9" s="159"/>
+      <c r="Q9" s="159"/>
+      <c r="R9" s="159"/>
+      <c r="S9" s="159"/>
+      <c r="T9" s="159"/>
+      <c r="U9" s="159"/>
+      <c r="V9" s="159"/>
+      <c r="W9" s="159"/>
+      <c r="X9" s="159"/>
+      <c r="Y9" s="159"/>
+      <c r="Z9" s="159"/>
+      <c r="AA9" s="159"/>
+      <c r="AB9" s="159"/>
+      <c r="AC9" s="159"/>
+      <c r="AD9" s="159"/>
+      <c r="AE9" s="159"/>
+      <c r="AF9" s="159"/>
+      <c r="AG9" s="160"/>
     </row>
     <row r="10" spans="1:33" ht="6.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="76"/>
-      <c r="B10" s="76"/>
-      <c r="C10" s="76"/>
-      <c r="D10" s="76"/>
-      <c r="E10" s="76"/>
-      <c r="F10" s="76"/>
-      <c r="G10" s="76"/>
-      <c r="H10" s="76"/>
-      <c r="I10" s="76"/>
-      <c r="J10" s="76"/>
-      <c r="K10" s="76"/>
-      <c r="L10" s="76"/>
-      <c r="M10" s="76"/>
-      <c r="N10" s="76"/>
-      <c r="O10" s="76"/>
-      <c r="P10" s="76"/>
-      <c r="Q10" s="76"/>
-      <c r="R10" s="76"/>
-      <c r="S10" s="76"/>
-      <c r="T10" s="76"/>
-      <c r="U10" s="76"/>
-      <c r="V10" s="76"/>
-      <c r="W10" s="76"/>
-      <c r="X10" s="76"/>
-      <c r="Y10" s="76"/>
-      <c r="Z10" s="76"/>
-      <c r="AA10" s="76"/>
-      <c r="AB10" s="76"/>
-      <c r="AC10" s="76"/>
-      <c r="AD10" s="76"/>
-      <c r="AE10" s="76"/>
-      <c r="AF10" s="76"/>
-      <c r="AG10" s="76"/>
+      <c r="A10" s="150"/>
+      <c r="B10" s="150"/>
+      <c r="C10" s="150"/>
+      <c r="D10" s="150"/>
+      <c r="E10" s="150"/>
+      <c r="F10" s="150"/>
+      <c r="G10" s="150"/>
+      <c r="H10" s="150"/>
+      <c r="I10" s="150"/>
+      <c r="J10" s="150"/>
+      <c r="K10" s="150"/>
+      <c r="L10" s="150"/>
+      <c r="M10" s="150"/>
+      <c r="N10" s="150"/>
+      <c r="O10" s="150"/>
+      <c r="P10" s="150"/>
+      <c r="Q10" s="150"/>
+      <c r="R10" s="150"/>
+      <c r="S10" s="150"/>
+      <c r="T10" s="150"/>
+      <c r="U10" s="150"/>
+      <c r="V10" s="150"/>
+      <c r="W10" s="150"/>
+      <c r="X10" s="150"/>
+      <c r="Y10" s="150"/>
+      <c r="Z10" s="150"/>
+      <c r="AA10" s="150"/>
+      <c r="AB10" s="150"/>
+      <c r="AC10" s="150"/>
+      <c r="AD10" s="150"/>
+      <c r="AE10" s="150"/>
+      <c r="AF10" s="150"/>
+      <c r="AG10" s="150"/>
     </row>
     <row r="11" spans="1:33" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
-      <c r="B11" s="116" t="s">
+      <c r="B11" s="51" t="s">
         <v>3</v>
       </c>
-      <c r="C11" s="116"/>
-      <c r="D11" s="117"/>
+      <c r="C11" s="51"/>
+      <c r="D11" s="52"/>
       <c r="E11" s="3"/>
       <c r="F11" s="6"/>
       <c r="G11" s="118" t="s">
@@ -3180,21 +3196,21 @@
       <c r="AB11" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="AC11" s="77" t="s">
+      <c r="AC11" s="161" t="s">
         <v>4</v>
       </c>
-      <c r="AD11" s="77"/>
-      <c r="AE11" s="77"/>
-      <c r="AF11" s="77"/>
-      <c r="AG11" s="77"/>
+      <c r="AD11" s="161"/>
+      <c r="AE11" s="161"/>
+      <c r="AF11" s="161"/>
+      <c r="AG11" s="161"/>
     </row>
     <row r="12" spans="1:33" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
-      <c r="B12" s="116" t="s">
+      <c r="B12" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="116"/>
-      <c r="D12" s="117"/>
+      <c r="C12" s="51"/>
+      <c r="D12" s="52"/>
       <c r="E12" s="3" t="s">
         <v>29</v>
       </c>
@@ -3221,21 +3237,21 @@
       <c r="Z12" s="119"/>
       <c r="AA12" s="5"/>
       <c r="AB12" s="3"/>
-      <c r="AC12" s="77" t="s">
+      <c r="AC12" s="161" t="s">
         <v>13</v>
       </c>
-      <c r="AD12" s="77"/>
-      <c r="AE12" s="77"/>
-      <c r="AF12" s="77"/>
-      <c r="AG12" s="77"/>
+      <c r="AD12" s="161"/>
+      <c r="AE12" s="161"/>
+      <c r="AF12" s="161"/>
+      <c r="AG12" s="161"/>
     </row>
     <row r="13" spans="1:33" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
-      <c r="B13" s="116" t="s">
+      <c r="B13" s="51" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="116"/>
-      <c r="D13" s="117"/>
+      <c r="C13" s="51"/>
+      <c r="D13" s="52"/>
       <c r="E13" s="3" t="s">
         <v>29</v>
       </c>
@@ -3305,79 +3321,79 @@
     </row>
     <row r="15" spans="1:33" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
-      <c r="B15" s="180" t="s">
+      <c r="B15" s="176" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="181"/>
-      <c r="D15" s="181"/>
-      <c r="E15" s="181"/>
-      <c r="F15" s="181"/>
-      <c r="G15" s="181"/>
-      <c r="H15" s="181"/>
-      <c r="I15" s="181"/>
-      <c r="J15" s="181"/>
-      <c r="K15" s="181"/>
-      <c r="L15" s="181"/>
-      <c r="M15" s="181"/>
-      <c r="N15" s="181"/>
-      <c r="O15" s="181"/>
-      <c r="P15" s="181"/>
-      <c r="Q15" s="181"/>
-      <c r="R15" s="181"/>
-      <c r="S15" s="179"/>
-      <c r="T15" s="179"/>
-      <c r="U15" s="179"/>
-      <c r="V15" s="179"/>
-      <c r="W15" s="179"/>
-      <c r="X15" s="179"/>
-      <c r="Y15" s="179"/>
-      <c r="Z15" s="78" t="s">
+      <c r="C15" s="177"/>
+      <c r="D15" s="177"/>
+      <c r="E15" s="177"/>
+      <c r="F15" s="177"/>
+      <c r="G15" s="177"/>
+      <c r="H15" s="177"/>
+      <c r="I15" s="177"/>
+      <c r="J15" s="177"/>
+      <c r="K15" s="177"/>
+      <c r="L15" s="177"/>
+      <c r="M15" s="177"/>
+      <c r="N15" s="177"/>
+      <c r="O15" s="177"/>
+      <c r="P15" s="177"/>
+      <c r="Q15" s="177"/>
+      <c r="R15" s="177"/>
+      <c r="S15" s="178"/>
+      <c r="T15" s="178"/>
+      <c r="U15" s="178"/>
+      <c r="V15" s="178"/>
+      <c r="W15" s="178"/>
+      <c r="X15" s="178"/>
+      <c r="Y15" s="178"/>
+      <c r="Z15" s="180" t="s">
         <v>1</v>
       </c>
-      <c r="AA15" s="78"/>
-      <c r="AB15" s="78"/>
-      <c r="AC15" s="177"/>
-      <c r="AD15" s="177"/>
-      <c r="AE15" s="177"/>
-      <c r="AF15" s="177"/>
-      <c r="AG15" s="178"/>
-    </row>
-    <row r="16" spans="1:33" s="34" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AA15" s="180"/>
+      <c r="AB15" s="180"/>
+      <c r="AC15" s="182"/>
+      <c r="AD15" s="182"/>
+      <c r="AE15" s="182"/>
+      <c r="AF15" s="182"/>
+      <c r="AG15" s="183"/>
+    </row>
+    <row r="16" spans="1:33" s="34" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="33"/>
-      <c r="B16" s="192" t="s">
-        <v>31</v>
-      </c>
-      <c r="C16" s="193"/>
-      <c r="D16" s="193"/>
-      <c r="E16" s="193"/>
-      <c r="F16" s="193"/>
-      <c r="G16" s="193"/>
-      <c r="H16" s="193"/>
-      <c r="I16" s="193"/>
-      <c r="J16" s="193"/>
-      <c r="K16" s="193"/>
-      <c r="L16" s="193"/>
-      <c r="M16" s="193"/>
-      <c r="N16" s="193"/>
-      <c r="O16" s="193"/>
-      <c r="P16" s="193"/>
-      <c r="Q16" s="193"/>
-      <c r="R16" s="193"/>
-      <c r="S16" s="193"/>
-      <c r="T16" s="193"/>
-      <c r="U16" s="193"/>
-      <c r="V16" s="193"/>
-      <c r="W16" s="193"/>
-      <c r="X16" s="193"/>
-      <c r="Y16" s="193"/>
-      <c r="Z16" s="193"/>
-      <c r="AA16" s="193"/>
-      <c r="AB16" s="193"/>
-      <c r="AC16" s="193"/>
-      <c r="AD16" s="193"/>
-      <c r="AE16" s="193"/>
-      <c r="AF16" s="193"/>
-      <c r="AG16" s="194"/>
+      <c r="B16" s="174" t="s">
+        <v>197</v>
+      </c>
+      <c r="C16" s="175"/>
+      <c r="D16" s="175"/>
+      <c r="E16" s="175"/>
+      <c r="F16" s="175"/>
+      <c r="G16" s="175"/>
+      <c r="H16" s="175"/>
+      <c r="I16" s="175"/>
+      <c r="J16" s="175"/>
+      <c r="K16" s="175"/>
+      <c r="L16" s="175"/>
+      <c r="M16" s="175"/>
+      <c r="N16" s="175"/>
+      <c r="O16" s="175"/>
+      <c r="P16" s="175"/>
+      <c r="Q16" s="175"/>
+      <c r="R16" s="175"/>
+      <c r="S16" s="179"/>
+      <c r="T16" s="179"/>
+      <c r="U16" s="179"/>
+      <c r="V16" s="179"/>
+      <c r="W16" s="179"/>
+      <c r="X16" s="179"/>
+      <c r="Y16" s="179"/>
+      <c r="Z16" s="181"/>
+      <c r="AA16" s="181"/>
+      <c r="AB16" s="181"/>
+      <c r="AC16" s="184"/>
+      <c r="AD16" s="184"/>
+      <c r="AE16" s="184"/>
+      <c r="AF16" s="184"/>
+      <c r="AG16" s="185"/>
     </row>
     <row r="17" spans="1:33" s="11" customFormat="1" ht="6.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="10"/>
@@ -3451,44 +3467,44 @@
     </row>
     <row r="19" spans="1:33" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
-      <c r="B19" s="182" t="s">
+      <c r="B19" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="C19" s="183"/>
-      <c r="D19" s="184"/>
-      <c r="E19" s="50"/>
+      <c r="C19" s="54"/>
+      <c r="D19" s="55"/>
+      <c r="E19" s="49"/>
       <c r="F19" s="7"/>
       <c r="G19" s="20" t="s">
-        <v>44</v>
-      </c>
-      <c r="H19" s="187"/>
-      <c r="I19" s="187"/>
-      <c r="J19" s="187"/>
-      <c r="K19" s="187"/>
-      <c r="L19" s="187"/>
-      <c r="M19" s="187"/>
-      <c r="N19" s="188" t="s">
-        <v>36</v>
-      </c>
-      <c r="O19" s="188"/>
-      <c r="P19" s="188"/>
-      <c r="Q19" s="188"/>
-      <c r="R19" s="188"/>
-      <c r="S19" s="188"/>
-      <c r="T19" s="188"/>
-      <c r="U19" s="188"/>
-      <c r="V19" s="188"/>
-      <c r="W19" s="188"/>
-      <c r="X19" s="188"/>
-      <c r="Y19" s="188"/>
-      <c r="Z19" s="188"/>
-      <c r="AA19" s="188"/>
-      <c r="AB19" s="188"/>
-      <c r="AC19" s="188"/>
-      <c r="AD19" s="188"/>
-      <c r="AE19" s="188"/>
-      <c r="AF19" s="188"/>
-      <c r="AG19" s="189"/>
+        <v>43</v>
+      </c>
+      <c r="H19" s="58"/>
+      <c r="I19" s="58"/>
+      <c r="J19" s="58"/>
+      <c r="K19" s="58"/>
+      <c r="L19" s="58"/>
+      <c r="M19" s="58"/>
+      <c r="N19" s="59" t="s">
+        <v>35</v>
+      </c>
+      <c r="O19" s="59"/>
+      <c r="P19" s="59"/>
+      <c r="Q19" s="59"/>
+      <c r="R19" s="59"/>
+      <c r="S19" s="59"/>
+      <c r="T19" s="59"/>
+      <c r="U19" s="59"/>
+      <c r="V19" s="59"/>
+      <c r="W19" s="59"/>
+      <c r="X19" s="59"/>
+      <c r="Y19" s="59"/>
+      <c r="Z19" s="59"/>
+      <c r="AA19" s="59"/>
+      <c r="AB19" s="59"/>
+      <c r="AC19" s="59"/>
+      <c r="AD19" s="59"/>
+      <c r="AE19" s="59"/>
+      <c r="AF19" s="59"/>
+      <c r="AG19" s="60"/>
     </row>
     <row r="20" spans="1:33" s="11" customFormat="1" ht="8.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="10"/>
@@ -3597,44 +3613,44 @@
     </row>
     <row r="23" spans="1:33" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
-      <c r="B23" s="185" t="s">
-        <v>43</v>
-      </c>
-      <c r="C23" s="186"/>
-      <c r="D23" s="186"/>
-      <c r="E23" s="51"/>
+      <c r="B23" s="56" t="s">
+        <v>42</v>
+      </c>
+      <c r="C23" s="57"/>
+      <c r="D23" s="57"/>
+      <c r="E23" s="50"/>
       <c r="F23" s="38"/>
-      <c r="G23" s="190" t="s">
-        <v>47</v>
-      </c>
-      <c r="H23" s="190"/>
-      <c r="I23" s="190"/>
-      <c r="J23" s="190"/>
-      <c r="K23" s="190"/>
-      <c r="L23" s="190"/>
-      <c r="M23" s="190"/>
-      <c r="N23" s="186" t="s">
+      <c r="G23" s="61" t="s">
+        <v>46</v>
+      </c>
+      <c r="H23" s="61"/>
+      <c r="I23" s="61"/>
+      <c r="J23" s="61"/>
+      <c r="K23" s="61"/>
+      <c r="L23" s="61"/>
+      <c r="M23" s="61"/>
+      <c r="N23" s="57" t="s">
         <v>6</v>
       </c>
-      <c r="O23" s="186"/>
-      <c r="P23" s="186"/>
-      <c r="Q23" s="186"/>
-      <c r="R23" s="186"/>
-      <c r="S23" s="186"/>
-      <c r="T23" s="186"/>
-      <c r="U23" s="186"/>
-      <c r="V23" s="186"/>
-      <c r="W23" s="186"/>
-      <c r="X23" s="186"/>
-      <c r="Y23" s="186"/>
-      <c r="Z23" s="186"/>
-      <c r="AA23" s="186"/>
-      <c r="AB23" s="186"/>
-      <c r="AC23" s="186"/>
-      <c r="AD23" s="186"/>
-      <c r="AE23" s="186"/>
-      <c r="AF23" s="186"/>
-      <c r="AG23" s="191"/>
+      <c r="O23" s="57"/>
+      <c r="P23" s="57"/>
+      <c r="Q23" s="57"/>
+      <c r="R23" s="57"/>
+      <c r="S23" s="57"/>
+      <c r="T23" s="57"/>
+      <c r="U23" s="57"/>
+      <c r="V23" s="57"/>
+      <c r="W23" s="57"/>
+      <c r="X23" s="57"/>
+      <c r="Y23" s="57"/>
+      <c r="Z23" s="57"/>
+      <c r="AA23" s="57"/>
+      <c r="AB23" s="57"/>
+      <c r="AC23" s="57"/>
+      <c r="AD23" s="57"/>
+      <c r="AE23" s="57"/>
+      <c r="AF23" s="57"/>
+      <c r="AG23" s="62"/>
     </row>
     <row r="24" spans="1:33" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
@@ -3673,7 +3689,7 @@
     </row>
     <row r="25" spans="1:33" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="132" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C25" s="133"/>
       <c r="D25" s="133"/>
@@ -3724,7 +3740,7 @@
     <row r="26" spans="1:33" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="32"/>
       <c r="B26" s="128" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C26" s="129"/>
       <c r="D26" s="129"/>
@@ -3735,7 +3751,7 @@
       <c r="I26" s="129"/>
       <c r="J26" s="47"/>
       <c r="K26" s="124" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L26" s="124"/>
       <c r="M26" s="124"/>
@@ -3762,276 +3778,276 @@
     </row>
     <row r="27" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
-      <c r="B27" s="159" t="s">
+      <c r="B27" s="66" t="s">
         <v>16</v>
       </c>
-      <c r="C27" s="160"/>
-      <c r="D27" s="160"/>
-      <c r="E27" s="160"/>
-      <c r="F27" s="160"/>
-      <c r="G27" s="160"/>
-      <c r="H27" s="160"/>
-      <c r="I27" s="160"/>
-      <c r="J27" s="160"/>
-      <c r="K27" s="160"/>
-      <c r="L27" s="160"/>
-      <c r="M27" s="160"/>
-      <c r="N27" s="160"/>
-      <c r="O27" s="160"/>
-      <c r="P27" s="160"/>
-      <c r="Q27" s="160"/>
-      <c r="R27" s="161"/>
-      <c r="S27" s="159" t="s">
+      <c r="C27" s="67"/>
+      <c r="D27" s="67"/>
+      <c r="E27" s="67"/>
+      <c r="F27" s="67"/>
+      <c r="G27" s="67"/>
+      <c r="H27" s="67"/>
+      <c r="I27" s="67"/>
+      <c r="J27" s="67"/>
+      <c r="K27" s="67"/>
+      <c r="L27" s="67"/>
+      <c r="M27" s="67"/>
+      <c r="N27" s="67"/>
+      <c r="O27" s="67"/>
+      <c r="P27" s="67"/>
+      <c r="Q27" s="67"/>
+      <c r="R27" s="68"/>
+      <c r="S27" s="66" t="s">
         <v>17</v>
       </c>
-      <c r="T27" s="160"/>
-      <c r="U27" s="160"/>
-      <c r="V27" s="160"/>
-      <c r="W27" s="160"/>
-      <c r="X27" s="160"/>
-      <c r="Y27" s="160"/>
-      <c r="Z27" s="161"/>
-      <c r="AA27" s="159" t="s">
+      <c r="T27" s="67"/>
+      <c r="U27" s="67"/>
+      <c r="V27" s="67"/>
+      <c r="W27" s="67"/>
+      <c r="X27" s="67"/>
+      <c r="Y27" s="67"/>
+      <c r="Z27" s="68"/>
+      <c r="AA27" s="66" t="s">
         <v>18</v>
       </c>
-      <c r="AB27" s="160"/>
-      <c r="AC27" s="160"/>
-      <c r="AD27" s="161"/>
-      <c r="AE27" s="159" t="s">
+      <c r="AB27" s="67"/>
+      <c r="AC27" s="67"/>
+      <c r="AD27" s="68"/>
+      <c r="AE27" s="66" t="s">
         <v>19</v>
       </c>
-      <c r="AF27" s="160"/>
-      <c r="AG27" s="161"/>
-    </row>
-    <row r="28" spans="1:33" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF27" s="67"/>
+      <c r="AG27" s="68"/>
+    </row>
+    <row r="28" spans="1:33" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
-      <c r="B28" s="171" t="s">
+      <c r="B28" s="186" t="s">
         <v>30</v>
       </c>
-      <c r="C28" s="171"/>
-      <c r="D28" s="171"/>
-      <c r="E28" s="171"/>
-      <c r="F28" s="171"/>
-      <c r="G28" s="171"/>
-      <c r="H28" s="171"/>
-      <c r="I28" s="171"/>
-      <c r="J28" s="171"/>
-      <c r="K28" s="171"/>
-      <c r="L28" s="171"/>
-      <c r="M28" s="171"/>
-      <c r="N28" s="171"/>
-      <c r="O28" s="171"/>
-      <c r="P28" s="171"/>
-      <c r="Q28" s="171"/>
-      <c r="R28" s="171"/>
-      <c r="S28" s="174" t="s">
+      <c r="C28" s="186"/>
+      <c r="D28" s="186"/>
+      <c r="E28" s="186"/>
+      <c r="F28" s="186"/>
+      <c r="G28" s="186"/>
+      <c r="H28" s="186"/>
+      <c r="I28" s="186"/>
+      <c r="J28" s="186"/>
+      <c r="K28" s="186"/>
+      <c r="L28" s="186"/>
+      <c r="M28" s="186"/>
+      <c r="N28" s="186"/>
+      <c r="O28" s="186"/>
+      <c r="P28" s="186"/>
+      <c r="Q28" s="186"/>
+      <c r="R28" s="186"/>
+      <c r="S28" s="63" t="s">
         <v>30</v>
       </c>
-      <c r="T28" s="174"/>
-      <c r="U28" s="165" t="s">
+      <c r="T28" s="63"/>
+      <c r="U28" s="189" t="s">
         <v>30</v>
       </c>
-      <c r="V28" s="165"/>
-      <c r="W28" s="165"/>
-      <c r="X28" s="165"/>
-      <c r="Y28" s="165"/>
-      <c r="Z28" s="165"/>
-      <c r="AA28" s="168" t="s">
+      <c r="V28" s="189"/>
+      <c r="W28" s="189"/>
+      <c r="X28" s="189"/>
+      <c r="Y28" s="189"/>
+      <c r="Z28" s="189"/>
+      <c r="AA28" s="83" t="s">
         <v>30</v>
       </c>
-      <c r="AB28" s="168"/>
-      <c r="AC28" s="168"/>
-      <c r="AD28" s="168"/>
-      <c r="AE28" s="82" t="s">
+      <c r="AB28" s="83"/>
+      <c r="AC28" s="83"/>
+      <c r="AD28" s="83"/>
+      <c r="AE28" s="165" t="s">
         <v>30</v>
       </c>
-      <c r="AF28" s="82"/>
-      <c r="AG28" s="82"/>
-    </row>
-    <row r="29" spans="1:33" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF28" s="165"/>
+      <c r="AG28" s="165"/>
+    </row>
+    <row r="29" spans="1:33" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
-      <c r="B29" s="172" t="s">
+      <c r="B29" s="187" t="s">
         <v>30</v>
       </c>
-      <c r="C29" s="172"/>
-      <c r="D29" s="172"/>
-      <c r="E29" s="172"/>
-      <c r="F29" s="172"/>
-      <c r="G29" s="172"/>
-      <c r="H29" s="172"/>
-      <c r="I29" s="172"/>
-      <c r="J29" s="172"/>
-      <c r="K29" s="172"/>
-      <c r="L29" s="172"/>
-      <c r="M29" s="172"/>
-      <c r="N29" s="172"/>
-      <c r="O29" s="172"/>
-      <c r="P29" s="172"/>
-      <c r="Q29" s="172"/>
-      <c r="R29" s="172"/>
-      <c r="S29" s="175" t="s">
+      <c r="C29" s="187"/>
+      <c r="D29" s="187"/>
+      <c r="E29" s="187"/>
+      <c r="F29" s="187"/>
+      <c r="G29" s="187"/>
+      <c r="H29" s="187"/>
+      <c r="I29" s="187"/>
+      <c r="J29" s="187"/>
+      <c r="K29" s="187"/>
+      <c r="L29" s="187"/>
+      <c r="M29" s="187"/>
+      <c r="N29" s="187"/>
+      <c r="O29" s="187"/>
+      <c r="P29" s="187"/>
+      <c r="Q29" s="187"/>
+      <c r="R29" s="187"/>
+      <c r="S29" s="64" t="s">
         <v>30</v>
       </c>
-      <c r="T29" s="175"/>
-      <c r="U29" s="166" t="s">
+      <c r="T29" s="64"/>
+      <c r="U29" s="190" t="s">
         <v>30</v>
       </c>
-      <c r="V29" s="166"/>
-      <c r="W29" s="166"/>
-      <c r="X29" s="166"/>
-      <c r="Y29" s="166"/>
-      <c r="Z29" s="166"/>
-      <c r="AA29" s="169" t="s">
+      <c r="V29" s="190"/>
+      <c r="W29" s="190"/>
+      <c r="X29" s="190"/>
+      <c r="Y29" s="190"/>
+      <c r="Z29" s="190"/>
+      <c r="AA29" s="84" t="s">
         <v>30</v>
       </c>
-      <c r="AB29" s="169"/>
-      <c r="AC29" s="169"/>
-      <c r="AD29" s="169"/>
-      <c r="AE29" s="134" t="s">
+      <c r="AB29" s="84"/>
+      <c r="AC29" s="84"/>
+      <c r="AD29" s="84"/>
+      <c r="AE29" s="69" t="s">
         <v>30</v>
       </c>
-      <c r="AF29" s="134"/>
-      <c r="AG29" s="134"/>
-    </row>
-    <row r="30" spans="1:33" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF29" s="69"/>
+      <c r="AG29" s="69"/>
+    </row>
+    <row r="30" spans="1:33" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
-      <c r="B30" s="172" t="s">
+      <c r="B30" s="187" t="s">
         <v>30</v>
       </c>
-      <c r="C30" s="172"/>
-      <c r="D30" s="172"/>
-      <c r="E30" s="172"/>
-      <c r="F30" s="172"/>
-      <c r="G30" s="172"/>
-      <c r="H30" s="172"/>
-      <c r="I30" s="172"/>
-      <c r="J30" s="172"/>
-      <c r="K30" s="172"/>
-      <c r="L30" s="172"/>
-      <c r="M30" s="172"/>
-      <c r="N30" s="172"/>
-      <c r="O30" s="172"/>
-      <c r="P30" s="172"/>
-      <c r="Q30" s="172"/>
-      <c r="R30" s="172"/>
-      <c r="S30" s="175" t="s">
+      <c r="C30" s="187"/>
+      <c r="D30" s="187"/>
+      <c r="E30" s="187"/>
+      <c r="F30" s="187"/>
+      <c r="G30" s="187"/>
+      <c r="H30" s="187"/>
+      <c r="I30" s="187"/>
+      <c r="J30" s="187"/>
+      <c r="K30" s="187"/>
+      <c r="L30" s="187"/>
+      <c r="M30" s="187"/>
+      <c r="N30" s="187"/>
+      <c r="O30" s="187"/>
+      <c r="P30" s="187"/>
+      <c r="Q30" s="187"/>
+      <c r="R30" s="187"/>
+      <c r="S30" s="64" t="s">
         <v>30</v>
       </c>
-      <c r="T30" s="175"/>
-      <c r="U30" s="166" t="s">
+      <c r="T30" s="64"/>
+      <c r="U30" s="190" t="s">
         <v>30</v>
       </c>
-      <c r="V30" s="166"/>
-      <c r="W30" s="166"/>
-      <c r="X30" s="166"/>
-      <c r="Y30" s="166"/>
-      <c r="Z30" s="166"/>
-      <c r="AA30" s="169" t="s">
+      <c r="V30" s="190"/>
+      <c r="W30" s="190"/>
+      <c r="X30" s="190"/>
+      <c r="Y30" s="190"/>
+      <c r="Z30" s="190"/>
+      <c r="AA30" s="84" t="s">
         <v>30</v>
       </c>
-      <c r="AB30" s="169"/>
-      <c r="AC30" s="169"/>
-      <c r="AD30" s="169"/>
-      <c r="AE30" s="134" t="s">
+      <c r="AB30" s="84"/>
+      <c r="AC30" s="84"/>
+      <c r="AD30" s="84"/>
+      <c r="AE30" s="69" t="s">
         <v>30</v>
       </c>
-      <c r="AF30" s="134"/>
-      <c r="AG30" s="134"/>
-    </row>
-    <row r="31" spans="1:33" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF30" s="69"/>
+      <c r="AG30" s="69"/>
+    </row>
+    <row r="31" spans="1:33" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
-      <c r="B31" s="172" t="s">
+      <c r="B31" s="187" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="172"/>
-      <c r="D31" s="172"/>
-      <c r="E31" s="172"/>
-      <c r="F31" s="172"/>
-      <c r="G31" s="172"/>
-      <c r="H31" s="172"/>
-      <c r="I31" s="172"/>
-      <c r="J31" s="172"/>
-      <c r="K31" s="172"/>
-      <c r="L31" s="172"/>
-      <c r="M31" s="172"/>
-      <c r="N31" s="172"/>
-      <c r="O31" s="172"/>
-      <c r="P31" s="172"/>
-      <c r="Q31" s="172"/>
-      <c r="R31" s="172"/>
-      <c r="S31" s="175" t="s">
+      <c r="C31" s="187"/>
+      <c r="D31" s="187"/>
+      <c r="E31" s="187"/>
+      <c r="F31" s="187"/>
+      <c r="G31" s="187"/>
+      <c r="H31" s="187"/>
+      <c r="I31" s="187"/>
+      <c r="J31" s="187"/>
+      <c r="K31" s="187"/>
+      <c r="L31" s="187"/>
+      <c r="M31" s="187"/>
+      <c r="N31" s="187"/>
+      <c r="O31" s="187"/>
+      <c r="P31" s="187"/>
+      <c r="Q31" s="187"/>
+      <c r="R31" s="187"/>
+      <c r="S31" s="64" t="s">
         <v>30</v>
       </c>
-      <c r="T31" s="175"/>
-      <c r="U31" s="166" t="s">
+      <c r="T31" s="64"/>
+      <c r="U31" s="190" t="s">
         <v>30</v>
       </c>
-      <c r="V31" s="166"/>
-      <c r="W31" s="166"/>
-      <c r="X31" s="166"/>
-      <c r="Y31" s="166"/>
-      <c r="Z31" s="166"/>
-      <c r="AA31" s="169" t="s">
+      <c r="V31" s="190"/>
+      <c r="W31" s="190"/>
+      <c r="X31" s="190"/>
+      <c r="Y31" s="190"/>
+      <c r="Z31" s="190"/>
+      <c r="AA31" s="84" t="s">
         <v>30</v>
       </c>
-      <c r="AB31" s="169"/>
-      <c r="AC31" s="169"/>
-      <c r="AD31" s="169"/>
-      <c r="AE31" s="134" t="s">
+      <c r="AB31" s="84"/>
+      <c r="AC31" s="84"/>
+      <c r="AD31" s="84"/>
+      <c r="AE31" s="69" t="s">
         <v>30</v>
       </c>
-      <c r="AF31" s="134"/>
-      <c r="AG31" s="134"/>
-    </row>
-    <row r="32" spans="1:33" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AF31" s="69"/>
+      <c r="AG31" s="69"/>
+    </row>
+    <row r="32" spans="1:33" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
-      <c r="B32" s="173" t="s">
+      <c r="B32" s="188" t="s">
         <v>30</v>
       </c>
-      <c r="C32" s="173"/>
-      <c r="D32" s="173"/>
-      <c r="E32" s="173"/>
-      <c r="F32" s="173"/>
-      <c r="G32" s="173"/>
-      <c r="H32" s="173"/>
-      <c r="I32" s="173"/>
-      <c r="J32" s="173"/>
-      <c r="K32" s="173"/>
-      <c r="L32" s="173"/>
-      <c r="M32" s="173"/>
-      <c r="N32" s="173"/>
-      <c r="O32" s="173"/>
-      <c r="P32" s="173"/>
-      <c r="Q32" s="173"/>
-      <c r="R32" s="173"/>
-      <c r="S32" s="176" t="s">
+      <c r="C32" s="188"/>
+      <c r="D32" s="188"/>
+      <c r="E32" s="188"/>
+      <c r="F32" s="188"/>
+      <c r="G32" s="188"/>
+      <c r="H32" s="188"/>
+      <c r="I32" s="188"/>
+      <c r="J32" s="188"/>
+      <c r="K32" s="188"/>
+      <c r="L32" s="188"/>
+      <c r="M32" s="188"/>
+      <c r="N32" s="188"/>
+      <c r="O32" s="188"/>
+      <c r="P32" s="188"/>
+      <c r="Q32" s="188"/>
+      <c r="R32" s="188"/>
+      <c r="S32" s="65" t="s">
         <v>30</v>
       </c>
-      <c r="T32" s="176"/>
-      <c r="U32" s="167" t="s">
+      <c r="T32" s="65"/>
+      <c r="U32" s="191" t="s">
         <v>30</v>
       </c>
-      <c r="V32" s="167"/>
-      <c r="W32" s="167"/>
-      <c r="X32" s="167"/>
-      <c r="Y32" s="167"/>
-      <c r="Z32" s="167"/>
-      <c r="AA32" s="170" t="s">
+      <c r="V32" s="191"/>
+      <c r="W32" s="191"/>
+      <c r="X32" s="191"/>
+      <c r="Y32" s="191"/>
+      <c r="Z32" s="191"/>
+      <c r="AA32" s="85" t="s">
         <v>30</v>
       </c>
-      <c r="AB32" s="170"/>
-      <c r="AC32" s="170"/>
-      <c r="AD32" s="170"/>
-      <c r="AE32" s="110" t="s">
+      <c r="AB32" s="85"/>
+      <c r="AC32" s="85"/>
+      <c r="AD32" s="85"/>
+      <c r="AE32" s="113" t="s">
         <v>30</v>
       </c>
-      <c r="AF32" s="110"/>
-      <c r="AG32" s="110"/>
+      <c r="AF32" s="113"/>
+      <c r="AG32" s="113"/>
     </row>
     <row r="33" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
       <c r="B33" s="122" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C33" s="123"/>
       <c r="D33" s="123"/>
@@ -4047,25 +4063,25 @@
       <c r="N33" s="123"/>
       <c r="O33" s="123"/>
       <c r="P33" s="123"/>
-      <c r="Q33" s="79" t="s">
-        <v>38</v>
-      </c>
-      <c r="R33" s="79"/>
-      <c r="S33" s="79"/>
-      <c r="T33" s="79"/>
-      <c r="U33" s="79"/>
-      <c r="V33" s="79"/>
-      <c r="W33" s="79"/>
-      <c r="X33" s="79"/>
-      <c r="Y33" s="79"/>
-      <c r="Z33" s="79"/>
-      <c r="AA33" s="79"/>
-      <c r="AB33" s="79"/>
-      <c r="AC33" s="79"/>
-      <c r="AD33" s="79"/>
-      <c r="AE33" s="79"/>
-      <c r="AF33" s="79"/>
-      <c r="AG33" s="80"/>
+      <c r="Q33" s="162" t="s">
+        <v>37</v>
+      </c>
+      <c r="R33" s="162"/>
+      <c r="S33" s="162"/>
+      <c r="T33" s="162"/>
+      <c r="U33" s="162"/>
+      <c r="V33" s="162"/>
+      <c r="W33" s="162"/>
+      <c r="X33" s="162"/>
+      <c r="Y33" s="162"/>
+      <c r="Z33" s="162"/>
+      <c r="AA33" s="162"/>
+      <c r="AB33" s="162"/>
+      <c r="AC33" s="162"/>
+      <c r="AD33" s="162"/>
+      <c r="AE33" s="162"/>
+      <c r="AF33" s="162"/>
+      <c r="AG33" s="163"/>
     </row>
     <row r="34" spans="1:33" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
@@ -4104,516 +4120,573 @@
     </row>
     <row r="35" spans="1:33" s="4" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
-      <c r="B35" s="150" t="s">
+      <c r="B35" s="74" t="s">
         <v>23</v>
       </c>
-      <c r="C35" s="151"/>
-      <c r="D35" s="151"/>
-      <c r="E35" s="151"/>
-      <c r="F35" s="151"/>
-      <c r="G35" s="151"/>
-      <c r="H35" s="151"/>
-      <c r="I35" s="151"/>
-      <c r="J35" s="151"/>
-      <c r="K35" s="151"/>
-      <c r="L35" s="151"/>
-      <c r="M35" s="151"/>
-      <c r="N35" s="151"/>
-      <c r="O35" s="151"/>
-      <c r="P35" s="152"/>
-      <c r="Q35" s="108" t="s">
+      <c r="C35" s="75"/>
+      <c r="D35" s="75"/>
+      <c r="E35" s="75"/>
+      <c r="F35" s="75"/>
+      <c r="G35" s="75"/>
+      <c r="H35" s="75"/>
+      <c r="I35" s="75"/>
+      <c r="J35" s="75"/>
+      <c r="K35" s="75"/>
+      <c r="L35" s="75"/>
+      <c r="M35" s="75"/>
+      <c r="N35" s="75"/>
+      <c r="O35" s="75"/>
+      <c r="P35" s="76"/>
+      <c r="Q35" s="111" t="s">
         <v>24</v>
       </c>
-      <c r="R35" s="109"/>
-      <c r="S35" s="150" t="s">
-        <v>41</v>
-      </c>
-      <c r="T35" s="151"/>
-      <c r="U35" s="151"/>
-      <c r="V35" s="151"/>
-      <c r="W35" s="151"/>
-      <c r="X35" s="151"/>
-      <c r="Y35" s="151"/>
-      <c r="Z35" s="151"/>
-      <c r="AA35" s="151"/>
-      <c r="AB35" s="151"/>
-      <c r="AC35" s="151"/>
-      <c r="AD35" s="151"/>
-      <c r="AE35" s="151"/>
-      <c r="AF35" s="151"/>
-      <c r="AG35" s="152"/>
+      <c r="R35" s="112"/>
+      <c r="S35" s="74" t="s">
+        <v>40</v>
+      </c>
+      <c r="T35" s="75"/>
+      <c r="U35" s="75"/>
+      <c r="V35" s="75"/>
+      <c r="W35" s="75"/>
+      <c r="X35" s="75"/>
+      <c r="Y35" s="75"/>
+      <c r="Z35" s="75"/>
+      <c r="AA35" s="75"/>
+      <c r="AB35" s="75"/>
+      <c r="AC35" s="75"/>
+      <c r="AD35" s="75"/>
+      <c r="AE35" s="75"/>
+      <c r="AF35" s="75"/>
+      <c r="AG35" s="76"/>
     </row>
     <row r="36" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
-      <c r="B36" s="153"/>
-      <c r="C36" s="154"/>
-      <c r="D36" s="154"/>
-      <c r="E36" s="154"/>
-      <c r="F36" s="154"/>
-      <c r="G36" s="154"/>
-      <c r="H36" s="154"/>
-      <c r="I36" s="154"/>
-      <c r="J36" s="154"/>
-      <c r="K36" s="154"/>
-      <c r="L36" s="154"/>
-      <c r="M36" s="154"/>
-      <c r="N36" s="154"/>
-      <c r="O36" s="154"/>
-      <c r="P36" s="155"/>
-      <c r="Q36" s="108"/>
-      <c r="R36" s="109"/>
-      <c r="S36" s="162"/>
-      <c r="T36" s="163"/>
-      <c r="U36" s="163"/>
-      <c r="V36" s="163"/>
-      <c r="W36" s="163"/>
-      <c r="X36" s="163"/>
-      <c r="Y36" s="163"/>
-      <c r="Z36" s="163"/>
-      <c r="AA36" s="163"/>
-      <c r="AB36" s="163"/>
-      <c r="AC36" s="163"/>
-      <c r="AD36" s="163"/>
-      <c r="AE36" s="163"/>
-      <c r="AF36" s="163"/>
-      <c r="AG36" s="164"/>
-    </row>
-    <row r="37" spans="1:33" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B36" s="105"/>
+      <c r="C36" s="106"/>
+      <c r="D36" s="106"/>
+      <c r="E36" s="106"/>
+      <c r="F36" s="106"/>
+      <c r="G36" s="106"/>
+      <c r="H36" s="106"/>
+      <c r="I36" s="106"/>
+      <c r="J36" s="106"/>
+      <c r="K36" s="106"/>
+      <c r="L36" s="106"/>
+      <c r="M36" s="106"/>
+      <c r="N36" s="106"/>
+      <c r="O36" s="106"/>
+      <c r="P36" s="107"/>
+      <c r="Q36" s="111"/>
+      <c r="R36" s="112"/>
+      <c r="S36" s="77"/>
+      <c r="T36" s="78"/>
+      <c r="U36" s="78"/>
+      <c r="V36" s="78"/>
+      <c r="W36" s="78"/>
+      <c r="X36" s="78"/>
+      <c r="Y36" s="78"/>
+      <c r="Z36" s="78"/>
+      <c r="AA36" s="78"/>
+      <c r="AB36" s="78"/>
+      <c r="AC36" s="78"/>
+      <c r="AD36" s="78"/>
+      <c r="AE36" s="78"/>
+      <c r="AF36" s="78"/>
+      <c r="AG36" s="79"/>
+    </row>
+    <row r="37" spans="1:33" ht="125.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
-      <c r="B37" s="156"/>
-      <c r="C37" s="157"/>
-      <c r="D37" s="157"/>
-      <c r="E37" s="157"/>
-      <c r="F37" s="157"/>
-      <c r="G37" s="157"/>
-      <c r="H37" s="157"/>
-      <c r="I37" s="157"/>
-      <c r="J37" s="157"/>
-      <c r="K37" s="157"/>
-      <c r="L37" s="157"/>
-      <c r="M37" s="157"/>
-      <c r="N37" s="157"/>
-      <c r="O37" s="157"/>
-      <c r="P37" s="158"/>
-      <c r="Q37" s="108"/>
-      <c r="R37" s="109"/>
-      <c r="S37" s="156"/>
-      <c r="T37" s="157"/>
-      <c r="U37" s="157"/>
-      <c r="V37" s="157"/>
-      <c r="W37" s="157"/>
-      <c r="X37" s="157"/>
-      <c r="Y37" s="157"/>
-      <c r="Z37" s="157"/>
-      <c r="AA37" s="157"/>
-      <c r="AB37" s="157"/>
-      <c r="AC37" s="157"/>
-      <c r="AD37" s="157"/>
-      <c r="AE37" s="157"/>
-      <c r="AF37" s="157"/>
-      <c r="AG37" s="158"/>
+      <c r="B37" s="80"/>
+      <c r="C37" s="81"/>
+      <c r="D37" s="81"/>
+      <c r="E37" s="81"/>
+      <c r="F37" s="81"/>
+      <c r="G37" s="81"/>
+      <c r="H37" s="81"/>
+      <c r="I37" s="81"/>
+      <c r="J37" s="81"/>
+      <c r="K37" s="81"/>
+      <c r="L37" s="81"/>
+      <c r="M37" s="81"/>
+      <c r="N37" s="81"/>
+      <c r="O37" s="81"/>
+      <c r="P37" s="82"/>
+      <c r="Q37" s="111"/>
+      <c r="R37" s="112"/>
+      <c r="S37" s="80"/>
+      <c r="T37" s="81"/>
+      <c r="U37" s="81"/>
+      <c r="V37" s="81"/>
+      <c r="W37" s="81"/>
+      <c r="X37" s="81"/>
+      <c r="Y37" s="81"/>
+      <c r="Z37" s="81"/>
+      <c r="AA37" s="81"/>
+      <c r="AB37" s="81"/>
+      <c r="AC37" s="81"/>
+      <c r="AD37" s="81"/>
+      <c r="AE37" s="81"/>
+      <c r="AF37" s="81"/>
+      <c r="AG37" s="82"/>
     </row>
     <row r="38" spans="1:33" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
-      <c r="B38" s="60" t="s">
+      <c r="B38" s="101" t="s">
         <v>25</v>
       </c>
-      <c r="C38" s="61"/>
-      <c r="D38" s="62"/>
-      <c r="E38" s="62"/>
-      <c r="F38" s="62"/>
-      <c r="G38" s="62"/>
-      <c r="H38" s="62"/>
-      <c r="I38" s="62"/>
-      <c r="J38" s="62"/>
-      <c r="K38" s="62"/>
-      <c r="L38" s="62"/>
-      <c r="M38" s="62"/>
-      <c r="N38" s="62"/>
-      <c r="O38" s="62"/>
-      <c r="P38" s="63"/>
-      <c r="Q38" s="108"/>
-      <c r="R38" s="109"/>
-      <c r="S38" s="60" t="s">
+      <c r="C38" s="102"/>
+      <c r="D38" s="70"/>
+      <c r="E38" s="70"/>
+      <c r="F38" s="70"/>
+      <c r="G38" s="70"/>
+      <c r="H38" s="70"/>
+      <c r="I38" s="70"/>
+      <c r="J38" s="70"/>
+      <c r="K38" s="70"/>
+      <c r="L38" s="70"/>
+      <c r="M38" s="70"/>
+      <c r="N38" s="70"/>
+      <c r="O38" s="70"/>
+      <c r="P38" s="71"/>
+      <c r="Q38" s="111"/>
+      <c r="R38" s="112"/>
+      <c r="S38" s="101" t="s">
         <v>25</v>
       </c>
-      <c r="T38" s="61"/>
-      <c r="U38" s="62"/>
-      <c r="V38" s="62"/>
-      <c r="W38" s="62"/>
-      <c r="X38" s="62"/>
-      <c r="Y38" s="62"/>
-      <c r="Z38" s="62"/>
-      <c r="AA38" s="62"/>
-      <c r="AB38" s="62"/>
-      <c r="AC38" s="62"/>
-      <c r="AD38" s="62"/>
-      <c r="AE38" s="62"/>
-      <c r="AF38" s="62"/>
-      <c r="AG38" s="63"/>
+      <c r="T38" s="102"/>
+      <c r="U38" s="70"/>
+      <c r="V38" s="70"/>
+      <c r="W38" s="70"/>
+      <c r="X38" s="70"/>
+      <c r="Y38" s="70"/>
+      <c r="Z38" s="70"/>
+      <c r="AA38" s="70"/>
+      <c r="AB38" s="70"/>
+      <c r="AC38" s="70"/>
+      <c r="AD38" s="70"/>
+      <c r="AE38" s="70"/>
+      <c r="AF38" s="70"/>
+      <c r="AG38" s="71"/>
     </row>
     <row r="39" spans="1:33" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
-      <c r="B39" s="58" t="s">
+      <c r="B39" s="103" t="s">
         <v>26</v>
       </c>
-      <c r="C39" s="59"/>
-      <c r="D39" s="64"/>
-      <c r="E39" s="64"/>
-      <c r="F39" s="64"/>
-      <c r="G39" s="64"/>
-      <c r="H39" s="64"/>
-      <c r="I39" s="64"/>
-      <c r="J39" s="64"/>
-      <c r="K39" s="64"/>
-      <c r="L39" s="64"/>
-      <c r="M39" s="64"/>
-      <c r="N39" s="64"/>
-      <c r="O39" s="64"/>
-      <c r="P39" s="65"/>
-      <c r="Q39" s="108"/>
-      <c r="R39" s="109"/>
-      <c r="S39" s="58" t="s">
+      <c r="C39" s="104"/>
+      <c r="D39" s="72"/>
+      <c r="E39" s="72"/>
+      <c r="F39" s="72"/>
+      <c r="G39" s="72"/>
+      <c r="H39" s="72"/>
+      <c r="I39" s="72"/>
+      <c r="J39" s="72"/>
+      <c r="K39" s="72"/>
+      <c r="L39" s="72"/>
+      <c r="M39" s="72"/>
+      <c r="N39" s="72"/>
+      <c r="O39" s="72"/>
+      <c r="P39" s="73"/>
+      <c r="Q39" s="111"/>
+      <c r="R39" s="112"/>
+      <c r="S39" s="103" t="s">
         <v>26</v>
       </c>
-      <c r="T39" s="59"/>
-      <c r="U39" s="64"/>
-      <c r="V39" s="64"/>
-      <c r="W39" s="64"/>
-      <c r="X39" s="64"/>
-      <c r="Y39" s="64"/>
-      <c r="Z39" s="64"/>
-      <c r="AA39" s="64"/>
-      <c r="AB39" s="64"/>
-      <c r="AC39" s="64"/>
-      <c r="AD39" s="64"/>
-      <c r="AE39" s="64"/>
-      <c r="AF39" s="64"/>
-      <c r="AG39" s="65"/>
+      <c r="T39" s="104"/>
+      <c r="U39" s="72"/>
+      <c r="V39" s="72"/>
+      <c r="W39" s="72"/>
+      <c r="X39" s="72"/>
+      <c r="Y39" s="72"/>
+      <c r="Z39" s="72"/>
+      <c r="AA39" s="72"/>
+      <c r="AB39" s="72"/>
+      <c r="AC39" s="72"/>
+      <c r="AD39" s="72"/>
+      <c r="AE39" s="72"/>
+      <c r="AF39" s="72"/>
+      <c r="AG39" s="73"/>
     </row>
     <row r="40" spans="1:33" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="81"/>
-      <c r="B40" s="81"/>
-      <c r="C40" s="81"/>
-      <c r="D40" s="81"/>
-      <c r="E40" s="81"/>
-      <c r="F40" s="81"/>
-      <c r="G40" s="81"/>
-      <c r="H40" s="81"/>
-      <c r="I40" s="81"/>
-      <c r="J40" s="81"/>
-      <c r="K40" s="81"/>
-      <c r="L40" s="81"/>
-      <c r="M40" s="81"/>
-      <c r="N40" s="81"/>
-      <c r="O40" s="81"/>
-      <c r="P40" s="81"/>
-      <c r="Q40" s="81"/>
-      <c r="R40" s="81"/>
-      <c r="S40" s="81"/>
-      <c r="T40" s="81"/>
-      <c r="U40" s="81"/>
-      <c r="V40" s="81"/>
-      <c r="W40" s="81"/>
-      <c r="X40" s="81"/>
-      <c r="Y40" s="81"/>
-      <c r="Z40" s="81"/>
-      <c r="AA40" s="81"/>
-      <c r="AB40" s="81"/>
-      <c r="AC40" s="81"/>
-      <c r="AD40" s="81"/>
-      <c r="AE40" s="81"/>
-      <c r="AF40" s="81"/>
+      <c r="A40" s="164"/>
+      <c r="B40" s="164"/>
+      <c r="C40" s="164"/>
+      <c r="D40" s="164"/>
+      <c r="E40" s="164"/>
+      <c r="F40" s="164"/>
+      <c r="G40" s="164"/>
+      <c r="H40" s="164"/>
+      <c r="I40" s="164"/>
+      <c r="J40" s="164"/>
+      <c r="K40" s="164"/>
+      <c r="L40" s="164"/>
+      <c r="M40" s="164"/>
+      <c r="N40" s="164"/>
+      <c r="O40" s="164"/>
+      <c r="P40" s="164"/>
+      <c r="Q40" s="164"/>
+      <c r="R40" s="164"/>
+      <c r="S40" s="164"/>
+      <c r="T40" s="164"/>
+      <c r="U40" s="164"/>
+      <c r="V40" s="164"/>
+      <c r="W40" s="164"/>
+      <c r="X40" s="164"/>
+      <c r="Y40" s="164"/>
+      <c r="Z40" s="164"/>
+      <c r="AA40" s="164"/>
+      <c r="AB40" s="164"/>
+      <c r="AC40" s="164"/>
+      <c r="AD40" s="164"/>
+      <c r="AE40" s="164"/>
+      <c r="AF40" s="164"/>
       <c r="AG40" s="1"/>
     </row>
     <row r="41" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2"/>
-      <c r="B41" s="135"/>
-      <c r="C41" s="136"/>
-      <c r="D41" s="136"/>
-      <c r="E41" s="136"/>
-      <c r="F41" s="136"/>
-      <c r="G41" s="136"/>
-      <c r="H41" s="136"/>
-      <c r="I41" s="136"/>
-      <c r="J41" s="136"/>
-      <c r="K41" s="136"/>
-      <c r="L41" s="136"/>
-      <c r="M41" s="136"/>
-      <c r="N41" s="136"/>
-      <c r="O41" s="136"/>
-      <c r="P41" s="137"/>
-      <c r="Q41" s="108" t="s">
+      <c r="B41" s="86"/>
+      <c r="C41" s="87"/>
+      <c r="D41" s="87"/>
+      <c r="E41" s="87"/>
+      <c r="F41" s="87"/>
+      <c r="G41" s="87"/>
+      <c r="H41" s="87"/>
+      <c r="I41" s="87"/>
+      <c r="J41" s="87"/>
+      <c r="K41" s="87"/>
+      <c r="L41" s="87"/>
+      <c r="M41" s="87"/>
+      <c r="N41" s="87"/>
+      <c r="O41" s="87"/>
+      <c r="P41" s="88"/>
+      <c r="Q41" s="111" t="s">
         <v>24</v>
       </c>
-      <c r="R41" s="109"/>
-      <c r="S41" s="135"/>
-      <c r="T41" s="136"/>
-      <c r="U41" s="136"/>
-      <c r="V41" s="136"/>
-      <c r="W41" s="136"/>
-      <c r="X41" s="136"/>
-      <c r="Y41" s="136"/>
-      <c r="Z41" s="136"/>
-      <c r="AA41" s="136"/>
-      <c r="AB41" s="136"/>
-      <c r="AC41" s="136"/>
-      <c r="AD41" s="136"/>
-      <c r="AE41" s="136"/>
-      <c r="AF41" s="136"/>
-      <c r="AG41" s="137"/>
+      <c r="R41" s="112"/>
+      <c r="S41" s="86"/>
+      <c r="T41" s="87"/>
+      <c r="U41" s="87"/>
+      <c r="V41" s="87"/>
+      <c r="W41" s="87"/>
+      <c r="X41" s="87"/>
+      <c r="Y41" s="87"/>
+      <c r="Z41" s="87"/>
+      <c r="AA41" s="87"/>
+      <c r="AB41" s="87"/>
+      <c r="AC41" s="87"/>
+      <c r="AD41" s="87"/>
+      <c r="AE41" s="87"/>
+      <c r="AF41" s="87"/>
+      <c r="AG41" s="88"/>
     </row>
     <row r="42" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
-      <c r="B42" s="138" t="s">
+      <c r="B42" s="89" t="s">
+        <v>38</v>
+      </c>
+      <c r="C42" s="90"/>
+      <c r="D42" s="90"/>
+      <c r="E42" s="90"/>
+      <c r="F42" s="90"/>
+      <c r="G42" s="90"/>
+      <c r="H42" s="90"/>
+      <c r="I42" s="90"/>
+      <c r="J42" s="90"/>
+      <c r="K42" s="90"/>
+      <c r="L42" s="90"/>
+      <c r="M42" s="90"/>
+      <c r="N42" s="90"/>
+      <c r="O42" s="90"/>
+      <c r="P42" s="91"/>
+      <c r="Q42" s="111"/>
+      <c r="R42" s="112"/>
+      <c r="S42" s="95" t="s">
         <v>39</v>
       </c>
-      <c r="C42" s="139"/>
-      <c r="D42" s="139"/>
-      <c r="E42" s="139"/>
-      <c r="F42" s="139"/>
-      <c r="G42" s="139"/>
-      <c r="H42" s="139"/>
-      <c r="I42" s="139"/>
-      <c r="J42" s="139"/>
-      <c r="K42" s="139"/>
-      <c r="L42" s="139"/>
-      <c r="M42" s="139"/>
-      <c r="N42" s="139"/>
-      <c r="O42" s="139"/>
-      <c r="P42" s="140"/>
-      <c r="Q42" s="108"/>
-      <c r="R42" s="109"/>
-      <c r="S42" s="144" t="s">
-        <v>40</v>
-      </c>
-      <c r="T42" s="145"/>
-      <c r="U42" s="145"/>
-      <c r="V42" s="145"/>
-      <c r="W42" s="145"/>
-      <c r="X42" s="145"/>
-      <c r="Y42" s="145"/>
-      <c r="Z42" s="145"/>
-      <c r="AA42" s="145"/>
-      <c r="AB42" s="145"/>
-      <c r="AC42" s="145"/>
-      <c r="AD42" s="145"/>
-      <c r="AE42" s="145"/>
-      <c r="AF42" s="145"/>
-      <c r="AG42" s="146"/>
+      <c r="T42" s="96"/>
+      <c r="U42" s="96"/>
+      <c r="V42" s="96"/>
+      <c r="W42" s="96"/>
+      <c r="X42" s="96"/>
+      <c r="Y42" s="96"/>
+      <c r="Z42" s="96"/>
+      <c r="AA42" s="96"/>
+      <c r="AB42" s="96"/>
+      <c r="AC42" s="96"/>
+      <c r="AD42" s="96"/>
+      <c r="AE42" s="96"/>
+      <c r="AF42" s="96"/>
+      <c r="AG42" s="97"/>
     </row>
     <row r="43" spans="1:33" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
-      <c r="B43" s="141"/>
-      <c r="C43" s="142"/>
-      <c r="D43" s="142"/>
-      <c r="E43" s="142"/>
-      <c r="F43" s="142"/>
-      <c r="G43" s="142"/>
-      <c r="H43" s="142"/>
-      <c r="I43" s="142"/>
-      <c r="J43" s="142"/>
-      <c r="K43" s="142"/>
-      <c r="L43" s="142"/>
-      <c r="M43" s="142"/>
-      <c r="N43" s="142"/>
-      <c r="O43" s="142"/>
-      <c r="P43" s="143"/>
-      <c r="Q43" s="108"/>
-      <c r="R43" s="109"/>
-      <c r="S43" s="147"/>
-      <c r="T43" s="148"/>
-      <c r="U43" s="148"/>
-      <c r="V43" s="148"/>
-      <c r="W43" s="148"/>
-      <c r="X43" s="148"/>
-      <c r="Y43" s="148"/>
-      <c r="Z43" s="148"/>
-      <c r="AA43" s="148"/>
-      <c r="AB43" s="148"/>
-      <c r="AC43" s="148"/>
-      <c r="AD43" s="148"/>
-      <c r="AE43" s="148"/>
-      <c r="AF43" s="148"/>
-      <c r="AG43" s="149"/>
-    </row>
-    <row r="44" spans="1:33" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B43" s="92"/>
+      <c r="C43" s="93"/>
+      <c r="D43" s="93"/>
+      <c r="E43" s="93"/>
+      <c r="F43" s="93"/>
+      <c r="G43" s="93"/>
+      <c r="H43" s="93"/>
+      <c r="I43" s="93"/>
+      <c r="J43" s="93"/>
+      <c r="K43" s="93"/>
+      <c r="L43" s="93"/>
+      <c r="M43" s="93"/>
+      <c r="N43" s="93"/>
+      <c r="O43" s="93"/>
+      <c r="P43" s="94"/>
+      <c r="Q43" s="111"/>
+      <c r="R43" s="112"/>
+      <c r="S43" s="98"/>
+      <c r="T43" s="99"/>
+      <c r="U43" s="99"/>
+      <c r="V43" s="99"/>
+      <c r="W43" s="99"/>
+      <c r="X43" s="99"/>
+      <c r="Y43" s="99"/>
+      <c r="Z43" s="99"/>
+      <c r="AA43" s="99"/>
+      <c r="AB43" s="99"/>
+      <c r="AC43" s="99"/>
+      <c r="AD43" s="99"/>
+      <c r="AE43" s="99"/>
+      <c r="AF43" s="99"/>
+      <c r="AG43" s="100"/>
+    </row>
+    <row r="44" spans="1:33" ht="125.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
-      <c r="B44" s="105"/>
-      <c r="C44" s="106"/>
-      <c r="D44" s="106"/>
-      <c r="E44" s="106"/>
-      <c r="F44" s="106"/>
-      <c r="G44" s="106"/>
-      <c r="H44" s="106"/>
-      <c r="I44" s="106"/>
-      <c r="J44" s="106"/>
-      <c r="K44" s="106"/>
-      <c r="L44" s="106"/>
-      <c r="M44" s="106"/>
-      <c r="N44" s="106"/>
-      <c r="O44" s="106"/>
-      <c r="P44" s="107"/>
-      <c r="Q44" s="108"/>
-      <c r="R44" s="109"/>
-      <c r="S44" s="105"/>
-      <c r="T44" s="106"/>
-      <c r="U44" s="106"/>
-      <c r="V44" s="106"/>
-      <c r="W44" s="106"/>
-      <c r="X44" s="106"/>
-      <c r="Y44" s="106"/>
-      <c r="Z44" s="106"/>
-      <c r="AA44" s="106"/>
-      <c r="AB44" s="106"/>
-      <c r="AC44" s="106"/>
-      <c r="AD44" s="106"/>
-      <c r="AE44" s="106"/>
-      <c r="AF44" s="106"/>
-      <c r="AG44" s="107"/>
+      <c r="B44" s="108"/>
+      <c r="C44" s="109"/>
+      <c r="D44" s="109"/>
+      <c r="E44" s="109"/>
+      <c r="F44" s="109"/>
+      <c r="G44" s="109"/>
+      <c r="H44" s="109"/>
+      <c r="I44" s="109"/>
+      <c r="J44" s="109"/>
+      <c r="K44" s="109"/>
+      <c r="L44" s="109"/>
+      <c r="M44" s="109"/>
+      <c r="N44" s="109"/>
+      <c r="O44" s="109"/>
+      <c r="P44" s="110"/>
+      <c r="Q44" s="111"/>
+      <c r="R44" s="112"/>
+      <c r="S44" s="108"/>
+      <c r="T44" s="109"/>
+      <c r="U44" s="109"/>
+      <c r="V44" s="109"/>
+      <c r="W44" s="109"/>
+      <c r="X44" s="109"/>
+      <c r="Y44" s="109"/>
+      <c r="Z44" s="109"/>
+      <c r="AA44" s="109"/>
+      <c r="AB44" s="109"/>
+      <c r="AC44" s="109"/>
+      <c r="AD44" s="109"/>
+      <c r="AE44" s="109"/>
+      <c r="AF44" s="109"/>
+      <c r="AG44" s="110"/>
     </row>
     <row r="45" spans="1:33" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
-      <c r="B45" s="52" t="s">
+      <c r="B45" s="166" t="s">
         <v>27</v>
       </c>
-      <c r="C45" s="53"/>
-      <c r="D45" s="53"/>
-      <c r="E45" s="53"/>
-      <c r="F45" s="53"/>
-      <c r="G45" s="53"/>
-      <c r="H45" s="53"/>
-      <c r="I45" s="53"/>
-      <c r="J45" s="53"/>
-      <c r="K45" s="53"/>
-      <c r="L45" s="53"/>
-      <c r="M45" s="53"/>
-      <c r="N45" s="53"/>
-      <c r="O45" s="53"/>
-      <c r="P45" s="54"/>
-      <c r="Q45" s="108"/>
-      <c r="R45" s="109"/>
-      <c r="S45" s="55" t="s">
+      <c r="C45" s="167"/>
+      <c r="D45" s="167"/>
+      <c r="E45" s="167"/>
+      <c r="F45" s="167"/>
+      <c r="G45" s="167"/>
+      <c r="H45" s="167"/>
+      <c r="I45" s="167"/>
+      <c r="J45" s="167"/>
+      <c r="K45" s="167"/>
+      <c r="L45" s="167"/>
+      <c r="M45" s="167"/>
+      <c r="N45" s="167"/>
+      <c r="O45" s="167"/>
+      <c r="P45" s="168"/>
+      <c r="Q45" s="111"/>
+      <c r="R45" s="112"/>
+      <c r="S45" s="169" t="s">
         <v>28</v>
       </c>
-      <c r="T45" s="56"/>
-      <c r="U45" s="56"/>
-      <c r="V45" s="56"/>
-      <c r="W45" s="56"/>
-      <c r="X45" s="56"/>
-      <c r="Y45" s="56"/>
-      <c r="Z45" s="56"/>
-      <c r="AA45" s="56"/>
-      <c r="AB45" s="56"/>
-      <c r="AC45" s="56"/>
-      <c r="AD45" s="56"/>
-      <c r="AE45" s="56"/>
-      <c r="AF45" s="56"/>
-      <c r="AG45" s="57"/>
+      <c r="T45" s="170"/>
+      <c r="U45" s="170"/>
+      <c r="V45" s="170"/>
+      <c r="W45" s="170"/>
+      <c r="X45" s="170"/>
+      <c r="Y45" s="170"/>
+      <c r="Z45" s="170"/>
+      <c r="AA45" s="170"/>
+      <c r="AB45" s="170"/>
+      <c r="AC45" s="170"/>
+      <c r="AD45" s="170"/>
+      <c r="AE45" s="170"/>
+      <c r="AF45" s="170"/>
+      <c r="AG45" s="171"/>
     </row>
     <row r="46" spans="1:33" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
-      <c r="B46" s="60" t="s">
+      <c r="B46" s="101" t="s">
         <v>25</v>
       </c>
-      <c r="C46" s="61"/>
-      <c r="D46" s="62"/>
-      <c r="E46" s="62"/>
-      <c r="F46" s="62"/>
-      <c r="G46" s="62"/>
-      <c r="H46" s="62"/>
-      <c r="I46" s="62"/>
-      <c r="J46" s="62"/>
-      <c r="K46" s="62"/>
-      <c r="L46" s="62"/>
-      <c r="M46" s="62"/>
-      <c r="N46" s="62"/>
-      <c r="O46" s="62"/>
-      <c r="P46" s="63"/>
-      <c r="Q46" s="108"/>
-      <c r="R46" s="109"/>
-      <c r="S46" s="60" t="s">
+      <c r="C46" s="102"/>
+      <c r="D46" s="70"/>
+      <c r="E46" s="70"/>
+      <c r="F46" s="70"/>
+      <c r="G46" s="70"/>
+      <c r="H46" s="70"/>
+      <c r="I46" s="70"/>
+      <c r="J46" s="70"/>
+      <c r="K46" s="70"/>
+      <c r="L46" s="70"/>
+      <c r="M46" s="70"/>
+      <c r="N46" s="70"/>
+      <c r="O46" s="70"/>
+      <c r="P46" s="71"/>
+      <c r="Q46" s="111"/>
+      <c r="R46" s="112"/>
+      <c r="S46" s="101" t="s">
         <v>25</v>
       </c>
-      <c r="T46" s="61"/>
-      <c r="U46" s="62"/>
-      <c r="V46" s="62"/>
-      <c r="W46" s="62"/>
-      <c r="X46" s="62"/>
-      <c r="Y46" s="62"/>
-      <c r="Z46" s="62"/>
-      <c r="AA46" s="62"/>
-      <c r="AB46" s="62"/>
-      <c r="AC46" s="62"/>
-      <c r="AD46" s="62"/>
-      <c r="AE46" s="62"/>
-      <c r="AF46" s="62"/>
-      <c r="AG46" s="63"/>
+      <c r="T46" s="102"/>
+      <c r="U46" s="70"/>
+      <c r="V46" s="70"/>
+      <c r="W46" s="70"/>
+      <c r="X46" s="70"/>
+      <c r="Y46" s="70"/>
+      <c r="Z46" s="70"/>
+      <c r="AA46" s="70"/>
+      <c r="AB46" s="70"/>
+      <c r="AC46" s="70"/>
+      <c r="AD46" s="70"/>
+      <c r="AE46" s="70"/>
+      <c r="AF46" s="70"/>
+      <c r="AG46" s="71"/>
     </row>
     <row r="47" spans="1:33" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
-      <c r="B47" s="58" t="s">
+      <c r="B47" s="103" t="s">
         <v>26</v>
       </c>
-      <c r="C47" s="59"/>
-      <c r="D47" s="64"/>
-      <c r="E47" s="64"/>
-      <c r="F47" s="64"/>
-      <c r="G47" s="64"/>
-      <c r="H47" s="64"/>
-      <c r="I47" s="64"/>
-      <c r="J47" s="64"/>
-      <c r="K47" s="64"/>
-      <c r="L47" s="64"/>
-      <c r="M47" s="64"/>
-      <c r="N47" s="64"/>
-      <c r="O47" s="64"/>
-      <c r="P47" s="65"/>
-      <c r="Q47" s="108"/>
-      <c r="R47" s="109"/>
-      <c r="S47" s="58" t="s">
+      <c r="C47" s="104"/>
+      <c r="D47" s="72"/>
+      <c r="E47" s="72"/>
+      <c r="F47" s="72"/>
+      <c r="G47" s="72"/>
+      <c r="H47" s="72"/>
+      <c r="I47" s="72"/>
+      <c r="J47" s="72"/>
+      <c r="K47" s="72"/>
+      <c r="L47" s="72"/>
+      <c r="M47" s="72"/>
+      <c r="N47" s="72"/>
+      <c r="O47" s="72"/>
+      <c r="P47" s="73"/>
+      <c r="Q47" s="111"/>
+      <c r="R47" s="112"/>
+      <c r="S47" s="103" t="s">
         <v>26</v>
       </c>
-      <c r="T47" s="59"/>
-      <c r="U47" s="66"/>
-      <c r="V47" s="66"/>
-      <c r="W47" s="66"/>
-      <c r="X47" s="66"/>
-      <c r="Y47" s="66"/>
-      <c r="Z47" s="66"/>
-      <c r="AA47" s="66"/>
-      <c r="AB47" s="66"/>
-      <c r="AC47" s="66"/>
-      <c r="AD47" s="66"/>
-      <c r="AE47" s="66"/>
-      <c r="AF47" s="66"/>
-      <c r="AG47" s="67"/>
+      <c r="T47" s="104"/>
+      <c r="U47" s="172"/>
+      <c r="V47" s="172"/>
+      <c r="W47" s="172"/>
+      <c r="X47" s="172"/>
+      <c r="Y47" s="172"/>
+      <c r="Z47" s="172"/>
+      <c r="AA47" s="172"/>
+      <c r="AB47" s="172"/>
+      <c r="AC47" s="172"/>
+      <c r="AD47" s="172"/>
+      <c r="AE47" s="172"/>
+      <c r="AF47" s="172"/>
+      <c r="AG47" s="173"/>
     </row>
     <row r="54" ht="24.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
-  <mergeCells count="123">
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="AC15:AG15"/>
-    <mergeCell ref="S15:Y15"/>
-    <mergeCell ref="B15:R15"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="H19:M19"/>
-    <mergeCell ref="N19:AG19"/>
-    <mergeCell ref="G23:M23"/>
-    <mergeCell ref="N23:AG23"/>
-    <mergeCell ref="B16:AG16"/>
-    <mergeCell ref="B29:R29"/>
-    <mergeCell ref="B30:R30"/>
-    <mergeCell ref="B31:R31"/>
-    <mergeCell ref="B32:R32"/>
-    <mergeCell ref="S28:T28"/>
-    <mergeCell ref="S29:T29"/>
-    <mergeCell ref="S30:T30"/>
-    <mergeCell ref="S31:T31"/>
-    <mergeCell ref="S32:T32"/>
+  <mergeCells count="124">
+    <mergeCell ref="B45:P45"/>
+    <mergeCell ref="S45:AG45"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="D46:P46"/>
+    <mergeCell ref="D47:P47"/>
+    <mergeCell ref="U46:AG46"/>
+    <mergeCell ref="U47:AG47"/>
+    <mergeCell ref="S46:T46"/>
+    <mergeCell ref="S47:T47"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="D8:AG8"/>
+    <mergeCell ref="B9:AG9"/>
+    <mergeCell ref="A10:AG10"/>
+    <mergeCell ref="AC12:AG12"/>
+    <mergeCell ref="AC11:AG11"/>
+    <mergeCell ref="Q33:AG33"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="E40:G40"/>
+    <mergeCell ref="H40:I40"/>
+    <mergeCell ref="J40:K40"/>
+    <mergeCell ref="L40:M40"/>
+    <mergeCell ref="N40:O40"/>
+    <mergeCell ref="P40:Q40"/>
+    <mergeCell ref="AE40:AF40"/>
+    <mergeCell ref="R40:S40"/>
+    <mergeCell ref="T40:U40"/>
+    <mergeCell ref="V40:W40"/>
+    <mergeCell ref="X40:Y40"/>
+    <mergeCell ref="Z40:AB40"/>
+    <mergeCell ref="AC40:AD40"/>
+    <mergeCell ref="AE28:AG28"/>
+    <mergeCell ref="N1:AG1"/>
+    <mergeCell ref="N2:Q2"/>
+    <mergeCell ref="R2:AG2"/>
+    <mergeCell ref="N3:AG5"/>
+    <mergeCell ref="B1:M2"/>
+    <mergeCell ref="B3:M4"/>
+    <mergeCell ref="G6:X6"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="G7:P7"/>
+    <mergeCell ref="Y6:AG6"/>
+    <mergeCell ref="B44:P44"/>
+    <mergeCell ref="S44:AG44"/>
+    <mergeCell ref="Q35:R39"/>
+    <mergeCell ref="Q41:R47"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="AE32:AG32"/>
+    <mergeCell ref="B5:M5"/>
+    <mergeCell ref="Q7:S7"/>
+    <mergeCell ref="T7:AG7"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="G11:Z11"/>
+    <mergeCell ref="G12:Z12"/>
+    <mergeCell ref="G13:Z13"/>
+    <mergeCell ref="AB13:AG13"/>
+    <mergeCell ref="B33:P33"/>
+    <mergeCell ref="K26:AG26"/>
+    <mergeCell ref="L25:M25"/>
+    <mergeCell ref="B26:I26"/>
+    <mergeCell ref="P25:Q25"/>
+    <mergeCell ref="T25:X25"/>
+    <mergeCell ref="AB25:AG25"/>
+    <mergeCell ref="B25:I25"/>
+    <mergeCell ref="AE30:AG30"/>
+    <mergeCell ref="B41:P41"/>
+    <mergeCell ref="B42:P42"/>
+    <mergeCell ref="B43:P43"/>
+    <mergeCell ref="S41:AG41"/>
+    <mergeCell ref="S42:AG42"/>
+    <mergeCell ref="S43:AG43"/>
+    <mergeCell ref="S38:T38"/>
+    <mergeCell ref="S39:T39"/>
+    <mergeCell ref="B35:P36"/>
+    <mergeCell ref="B37:P37"/>
     <mergeCell ref="AE27:AG27"/>
     <mergeCell ref="AE29:AG29"/>
     <mergeCell ref="D38:P38"/>
@@ -4638,89 +4711,33 @@
     <mergeCell ref="AA31:AD31"/>
     <mergeCell ref="AA32:AD32"/>
     <mergeCell ref="B28:R28"/>
-    <mergeCell ref="B41:P41"/>
-    <mergeCell ref="B42:P42"/>
-    <mergeCell ref="B43:P43"/>
-    <mergeCell ref="S41:AG41"/>
-    <mergeCell ref="S42:AG42"/>
-    <mergeCell ref="S43:AG43"/>
-    <mergeCell ref="S38:T38"/>
-    <mergeCell ref="S39:T39"/>
-    <mergeCell ref="B35:P36"/>
-    <mergeCell ref="B37:P37"/>
-    <mergeCell ref="B44:P44"/>
-    <mergeCell ref="S44:AG44"/>
-    <mergeCell ref="Q35:R39"/>
-    <mergeCell ref="Q41:R47"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="AE32:AG32"/>
-    <mergeCell ref="B5:M5"/>
-    <mergeCell ref="Q7:S7"/>
-    <mergeCell ref="T7:AG7"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="G11:Z11"/>
-    <mergeCell ref="G12:Z12"/>
-    <mergeCell ref="G13:Z13"/>
-    <mergeCell ref="AB13:AG13"/>
-    <mergeCell ref="B33:P33"/>
-    <mergeCell ref="K26:AG26"/>
-    <mergeCell ref="L25:M25"/>
-    <mergeCell ref="B26:I26"/>
-    <mergeCell ref="P25:Q25"/>
-    <mergeCell ref="T25:X25"/>
-    <mergeCell ref="AB25:AG25"/>
-    <mergeCell ref="B25:I25"/>
-    <mergeCell ref="AE30:AG30"/>
-    <mergeCell ref="N1:AG1"/>
-    <mergeCell ref="N2:Q2"/>
-    <mergeCell ref="R2:AG2"/>
-    <mergeCell ref="N3:AG5"/>
-    <mergeCell ref="B1:M2"/>
-    <mergeCell ref="B3:M4"/>
-    <mergeCell ref="G6:X6"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B7:F7"/>
-    <mergeCell ref="G7:P7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="D8:AG8"/>
-    <mergeCell ref="B9:AG9"/>
-    <mergeCell ref="A10:AG10"/>
-    <mergeCell ref="AC12:AG12"/>
-    <mergeCell ref="AC11:AG11"/>
-    <mergeCell ref="Z15:AB15"/>
-    <mergeCell ref="Q33:AG33"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="E40:G40"/>
-    <mergeCell ref="H40:I40"/>
-    <mergeCell ref="J40:K40"/>
-    <mergeCell ref="L40:M40"/>
-    <mergeCell ref="N40:O40"/>
-    <mergeCell ref="P40:Q40"/>
-    <mergeCell ref="AE40:AF40"/>
-    <mergeCell ref="R40:S40"/>
-    <mergeCell ref="T40:U40"/>
-    <mergeCell ref="V40:W40"/>
-    <mergeCell ref="X40:Y40"/>
-    <mergeCell ref="Z40:AB40"/>
-    <mergeCell ref="AC40:AD40"/>
-    <mergeCell ref="AE28:AG28"/>
-    <mergeCell ref="B45:P45"/>
-    <mergeCell ref="S45:AG45"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="D46:P46"/>
-    <mergeCell ref="D47:P47"/>
-    <mergeCell ref="U46:AG46"/>
-    <mergeCell ref="U47:AG47"/>
-    <mergeCell ref="S46:T46"/>
-    <mergeCell ref="S47:T47"/>
+    <mergeCell ref="B29:R29"/>
+    <mergeCell ref="B30:R30"/>
+    <mergeCell ref="B31:R31"/>
+    <mergeCell ref="B32:R32"/>
+    <mergeCell ref="S28:T28"/>
+    <mergeCell ref="S29:T29"/>
+    <mergeCell ref="S30:T30"/>
+    <mergeCell ref="S31:T31"/>
+    <mergeCell ref="S32:T32"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B15:R15"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="H19:M19"/>
+    <mergeCell ref="N19:AG19"/>
+    <mergeCell ref="G23:M23"/>
+    <mergeCell ref="N23:AG23"/>
+    <mergeCell ref="B16:R16"/>
+    <mergeCell ref="S15:Y16"/>
+    <mergeCell ref="Z15:AB16"/>
+    <mergeCell ref="AC15:AG16"/>
   </mergeCells>
-  <phoneticPr fontId="16" type="noConversion"/>
+  <phoneticPr fontId="15" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.15748031496062992" right="0.15748031496062992" top="0.35433070866141736" bottom="0.35433070866141736" header="0.23622047244094491" footer="0.15748031496062992"/>
-  <pageSetup paperSize="9" scale="72" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="71" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddFooter>&amp;L&amp;"-,Italique"&amp;10LBo/VIGIE 2026</oddFooter>
   </headerFooter>
@@ -4729,12 +4746,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <scriptIds xmlns="http://schemas.microsoft.com/office/extensibility/maker/v1.0" id="script-ids-node-id">
   <scriptId id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F0176KMAHKB25D3ZMQHZ5CZCBZ22IEHSWLS:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9tYXJzZWlsbGVwb3J0LW15LnNoYXJlcG9pbnQuY29tLzp1Oi9nL3BlcnNvbmFsL2xhdXJlbnRfYm9oYm90X21hcnNlaWxsZS1wb3J0X2ZyL0VVSFhSN3l5Qjg5RmtRYzYwZ2g1V1hJQlZUdXF4ajdrenkwa0I2c0R1RVYwS2c"/>
   <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F0176KMAHISJHJEKOWIPRDZRJAPWYYADLK6:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9tYXJzZWlsbGVwb3J0LW15LnNoYXJlcG9pbnQuY29tLzp1Oi9nL3BlcnNvbmFsL2xhdXJlbnRfYm9oYm90X21hcnNlaWxsZS1wb3J0X2ZyL0VSSkowa1U2eUh4SG1LUVB0akFCclY0QmNqRC1JZnlfdy00cDZweDd1akVablE"/>
@@ -4742,16 +4753,13 @@
 </scriptIds>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A15EDE419BE4F64880B4C91CDDF245D8" ma:contentTypeVersion="4" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="7384b9ee12fa1f337ccf9a3feb43f0f2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="11f3f751-5cf8-4f05-a346-efdaa20acf12" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="80189908de78e9c0a30da25a41ecd7b9" ns2:_="">
     <xsd:import namespace="11f3f751-5cf8-4f05-a346-efdaa20acf12"/>
@@ -4895,7 +4903,25 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FFCC435E-9F5F-49FD-8CC7-C2246929C77B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/extensibility/maker/v1.0"/>
+    <ds:schemaRef ds:uri=""/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5CB41729-99EE-416A-81C7-6AA488F668EB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -4904,24 +4930,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FFCC435E-9F5F-49FD-8CC7-C2246929C77B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/extensibility/maker/v1.0"/>
-    <ds:schemaRef ds:uri=""/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F916078-60A3-4AA1-A4EE-7152721F381A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{046676A7-B87B-4BE6-8450-5088A25D540A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4937,4 +4946,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F916078-60A3-4AA1-A4EE-7152721F381A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>